<commit_message>
ATUALIZAÇÃO DE PLANILHA MARÇO - CHECKLIST 13/03 08:25
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA - LOCALIZAÇÃO DIARIA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161C0B09-DAAE-4CCA-B624-54B83E616804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C26D0BFB-C8E8-4FCF-B81E-F328437EA460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="368">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1140,6 +1140,9 @@
   </si>
   <si>
     <t>DATA DA CONFERENCIA: 13/03/2026</t>
+  </si>
+  <si>
+    <t>OPERADOR / CONTATO</t>
   </si>
 </sst>
 </file>
@@ -4211,7 +4214,7 @@
         <v>327</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>331</v>
+        <v>367</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>328</v>
@@ -4219,7 +4222,7 @@
       <c r="F6" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="1" t="s">
         <v>338</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA FROTA POTY: 16/03 09:15
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4506C780-EDF2-4266-BDA4-92512FC9D4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{990B19C2-4FA8-45A0-98B9-EA09FE2748EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
     <sheet name="13" sheetId="3" r:id="rId2"/>
+    <sheet name="16" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'13'!$A$6:$G$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'16'!$A$6:$G$170</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="387">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1143,6 +1145,65 @@
   </si>
   <si>
     <t>OPERADOR /CONTATO</t>
+  </si>
+  <si>
+    <t>Jardim do Mulato</t>
+  </si>
+  <si>
+    <t>Clodomiro Oliveira dos Santos / 
+Fábio da Silva Carvalho</t>
+  </si>
+  <si>
+    <t>Fábio da Silva Carvalho</t>
+  </si>
+  <si>
+    <t>OFICINA</t>
+  </si>
+  <si>
+    <t>CADOZ</t>
+  </si>
+  <si>
+    <t>TERESINA</t>
+  </si>
+  <si>
+    <t>SÃO FRANCISCO</t>
+  </si>
+  <si>
+    <t>FLORIANO</t>
+  </si>
+  <si>
+    <t>PORTO / N.S. REMÉDIOS</t>
+  </si>
+  <si>
+    <t>JOCA MARQUES / MADEIRO</t>
+  </si>
+  <si>
+    <t>PI 240 / ANTÔNIO ALMEIDA</t>
+  </si>
+  <si>
+    <t>PEDRO II</t>
+  </si>
+  <si>
+    <t>STATUS
+OFICINA/OPERACIONAL)</t>
+  </si>
+  <si>
+    <t>ÁGUA BRANCA</t>
+  </si>
+  <si>
+    <t>JADIM DO MULATO</t>
+  </si>
+  <si>
+    <t>JARDIM DO MULATO</t>
+  </si>
+  <si>
+    <t>JOAQUIM PIRES</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERENCIA: 16/03/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> José Mecias Dos Santos /  86995749413</t>
   </si>
 </sst>
 </file>
@@ -1198,7 +1259,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1226,6 +1287,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1284,7 +1351,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1312,6 +1379,9 @@
     <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1329,6 +1399,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF1FD59"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1414,6 +1489,59 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F8B8FC95-9A25-4539-B5D6-3AECDA9AAF4C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65B41B34-48E6-4834-BFF0-ACA23D7EBE16}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1780,45 +1908,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="13" t="s">
         <v>338</v>
       </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -3172,16 +3300,22 @@
       <c r="F103" s="4"/>
       <c r="G103" s="9"/>
     </row>
-    <row r="104" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A104" s="8" t="s">
         <v>193</v>
       </c>
       <c r="B104" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="C104" s="8"/>
-      <c r="D104" s="8"/>
-      <c r="E104" s="8"/>
+      <c r="C104" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="D104" s="8" t="s">
+        <v>369</v>
+      </c>
+      <c r="E104" s="8" t="s">
+        <v>370</v>
+      </c>
       <c r="F104" s="8"/>
       <c r="G104" s="10"/>
     </row>
@@ -4160,45 +4294,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="13" t="s">
         <v>365</v>
       </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -6512,6 +6646,2532 @@
       <c r="E170" s="4"/>
       <c r="F170" s="4"/>
       <c r="G170" s="9"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G170" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FE968AC-069D-4DBD-A367-7130F934BAB8}">
+  <dimension ref="A1:G170"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="39.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="38.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="13" t="s">
+        <v>385</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4"/>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="10"/>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G46" s="10"/>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="10"/>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="8"/>
+      <c r="G56" s="10"/>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="10"/>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="10"/>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8"/>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4"/>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10"/>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="9"/>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="8"/>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8"/>
+      <c r="F76" s="8"/>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4"/>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8"/>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="8"/>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10"/>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8"/>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8"/>
+      <c r="F84" s="8"/>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4"/>
+      <c r="D85" s="4"/>
+      <c r="E85" s="4"/>
+      <c r="F85" s="4"/>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8"/>
+      <c r="D86" s="8"/>
+      <c r="E86" s="8"/>
+      <c r="F86" s="8"/>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4"/>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
+      <c r="F87" s="4"/>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8"/>
+      <c r="D88" s="8"/>
+      <c r="E88" s="8"/>
+      <c r="F88" s="8"/>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4"/>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4"/>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8"/>
+      <c r="D90" s="8"/>
+      <c r="E90" s="8"/>
+      <c r="F90" s="8"/>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4"/>
+      <c r="D91" s="4"/>
+      <c r="E91" s="4"/>
+      <c r="F91" s="4"/>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8"/>
+      <c r="D92" s="8"/>
+      <c r="E92" s="8"/>
+      <c r="F92" s="8"/>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4"/>
+      <c r="E93" s="4"/>
+      <c r="F93" s="4"/>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8"/>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8"/>
+      <c r="F94" s="8"/>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+      <c r="F95" s="4"/>
+      <c r="G95" s="9"/>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="8"/>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8"/>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8"/>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8"/>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+      <c r="F105" s="4"/>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8"/>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8"/>
+      <c r="F106" s="8"/>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8"/>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8"/>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A112" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="C112" s="8"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="8"/>
+      <c r="G112" s="10"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A113" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E113" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="9"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C114" s="8"/>
+      <c r="D114" s="8"/>
+      <c r="E114" s="8"/>
+      <c r="F114" s="8"/>
+      <c r="G114" s="10"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A115" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C115" s="4"/>
+      <c r="D115" s="4"/>
+      <c r="E115" s="4"/>
+      <c r="F115" s="4"/>
+      <c r="G115" s="9"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A116" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C116" s="8"/>
+      <c r="D116" s="8"/>
+      <c r="E116" s="8"/>
+      <c r="F116" s="8"/>
+      <c r="G116" s="10"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C117" s="4"/>
+      <c r="D117" s="4"/>
+      <c r="E117" s="4"/>
+      <c r="F117" s="4"/>
+      <c r="G117" s="9"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B118" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C118" s="8"/>
+      <c r="D118" s="8"/>
+      <c r="E118" s="8"/>
+      <c r="F118" s="8"/>
+      <c r="G118" s="10"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C119" s="4"/>
+      <c r="D119" s="4"/>
+      <c r="E119" s="4"/>
+      <c r="F119" s="4"/>
+      <c r="G119" s="9"/>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C120" s="8"/>
+      <c r="D120" s="8"/>
+      <c r="E120" s="8"/>
+      <c r="F120" s="8"/>
+      <c r="G120" s="10"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C121" s="4"/>
+      <c r="D121" s="4"/>
+      <c r="E121" s="4"/>
+      <c r="F121" s="4"/>
+      <c r="G121" s="9"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B122" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C122" s="8"/>
+      <c r="D122" s="8"/>
+      <c r="E122" s="8"/>
+      <c r="F122" s="8"/>
+      <c r="G122" s="10"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C123" s="4"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
+      <c r="G123" s="9"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A124" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B124" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C124" s="8"/>
+      <c r="D124" s="8"/>
+      <c r="E124" s="8"/>
+      <c r="F124" s="8"/>
+      <c r="G124" s="10"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="D125" s="4"/>
+      <c r="E125" s="4"/>
+      <c r="F125" s="4"/>
+      <c r="G125" s="9"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C126" s="8"/>
+      <c r="D126" s="8"/>
+      <c r="E126" s="8"/>
+      <c r="F126" s="8"/>
+      <c r="G126" s="10"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A127" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E127" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G127" s="9"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A128" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C128" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="8"/>
+      <c r="E128" s="8"/>
+      <c r="F128" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G128" s="10"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A129" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="4"/>
+      <c r="E129" s="4"/>
+      <c r="F129" s="4"/>
+      <c r="G129" s="9"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="8"/>
+      <c r="E130" s="8"/>
+      <c r="F130" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G130" s="10"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A131" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C131" s="4"/>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+      <c r="G131" s="9"/>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D132" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F132" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D133" s="4"/>
+      <c r="E133" s="4"/>
+      <c r="F133" s="4"/>
+      <c r="G133" s="9"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C134" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D134" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F134" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="10"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E135" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G135" s="9"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A136" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C136" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D136" s="8"/>
+      <c r="E136" s="8"/>
+      <c r="F136" s="8"/>
+      <c r="G136" s="10"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A137" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E137" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="9"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A138" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C138" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D138" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F138" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="10"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D139" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E139" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G139" s="9"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A140" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C140" s="8"/>
+      <c r="D140" s="8"/>
+      <c r="E140" s="8"/>
+      <c r="F140" s="8"/>
+      <c r="G140" s="10"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A141" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C141" s="4"/>
+      <c r="D141" s="4"/>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="9"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A142" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C142" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="8"/>
+      <c r="E142" s="8"/>
+      <c r="F142" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G142" s="10"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4"/>
+      <c r="G143" s="9"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="8"/>
+      <c r="E144" s="8"/>
+      <c r="F144" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G144" s="10"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C145" s="4"/>
+      <c r="D145" s="4"/>
+      <c r="E145" s="4"/>
+      <c r="F145" s="4"/>
+      <c r="G145" s="9"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A146" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B146" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C146" s="8"/>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8"/>
+      <c r="G146" s="10"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A147" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="E147" s="4"/>
+      <c r="F147" s="4"/>
+      <c r="G147" s="9"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A148" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B148" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C148" s="8"/>
+      <c r="D148" s="8"/>
+      <c r="E148" s="8"/>
+      <c r="F148" s="8"/>
+      <c r="G148" s="10"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A149" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C149" s="4"/>
+      <c r="D149" s="4"/>
+      <c r="E149" s="4"/>
+      <c r="F149" s="4"/>
+      <c r="G149" s="9"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A150" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C150" s="8"/>
+      <c r="D150" s="8"/>
+      <c r="E150" s="8"/>
+      <c r="F150" s="8"/>
+      <c r="G150" s="10"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A151" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="9"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A152" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B152" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C152" s="8"/>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
+      <c r="F152" s="8"/>
+      <c r="G152" s="10"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A153" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C153" s="4"/>
+      <c r="D153" s="4"/>
+      <c r="E153" s="4"/>
+      <c r="F153" s="4"/>
+      <c r="G153" s="9"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A154" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C154" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="D154" s="8"/>
+      <c r="E154" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F154" s="8"/>
+      <c r="G154" s="10"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A155" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4"/>
+      <c r="G155" s="9"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A156" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C156" s="8"/>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8"/>
+      <c r="F156" s="8"/>
+      <c r="G156" s="10"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A157" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C157" s="4"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4"/>
+      <c r="G157" s="9"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A158" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B158" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C158" s="8"/>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8"/>
+      <c r="F158" s="8"/>
+      <c r="G158" s="10"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A159" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="9"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A160" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B160" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C160" s="8"/>
+      <c r="D160" s="8"/>
+      <c r="E160" s="8"/>
+      <c r="F160" s="8"/>
+      <c r="G160" s="10"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A161" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+      <c r="G161" s="9"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A162" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B162" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C162" s="8"/>
+      <c r="D162" s="8"/>
+      <c r="E162" s="8"/>
+      <c r="F162" s="8"/>
+      <c r="G162" s="10"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A163" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+      <c r="G163" s="9"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A164" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B164" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C164" s="8"/>
+      <c r="D164" s="8"/>
+      <c r="E164" s="8"/>
+      <c r="F164" s="8"/>
+      <c r="G164" s="10"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A165" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C165" s="4"/>
+      <c r="D165" s="4"/>
+      <c r="E165" s="4"/>
+      <c r="F165" s="4"/>
+      <c r="G165" s="9"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A166" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B166" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C166" s="8"/>
+      <c r="D166" s="8"/>
+      <c r="E166" s="8"/>
+      <c r="F166" s="8"/>
+      <c r="G166" s="10"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A167" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D167" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E167" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G167" s="9"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B168" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C168" s="8"/>
+      <c r="D168" s="8"/>
+      <c r="E168" s="8"/>
+      <c r="F168" s="8"/>
+      <c r="G168" s="10"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A169" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C169" s="4"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="9"/>
+    </row>
+    <row r="170" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A170" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B170" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C170" s="8"/>
+      <c r="D170" s="8"/>
+      <c r="E170" s="8"/>
+      <c r="F170" s="8"/>
+      <c r="G170" s="10"/>
     </row>
   </sheetData>
   <autoFilter ref="A6:G170" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA FROTA POTY: 16/03 09:40
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{990B19C2-4FA8-45A0-98B9-EA09FE2748EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C90CBD-B162-4F03-9C37-BC44CE7ECEA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="387">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -6744,10 +6744,10 @@
       <c r="B7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>373</v>
       </c>
+      <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4" t="s">
         <v>371</v>
@@ -6811,7 +6811,9 @@
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G11" s="9"/>
     </row>
     <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -6868,10 +6870,10 @@
       <c r="B15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4" t="s">
+      <c r="C15" s="4" t="s">
         <v>373</v>
       </c>
+      <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4" t="s">
         <v>371</v>
@@ -6991,7 +6993,9 @@
       <c r="E23" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="F23" s="4"/>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G23" s="9"/>
     </row>
     <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -7014,10 +7018,10 @@
       <c r="B25" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="4" t="s">
         <v>373</v>
       </c>
+      <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4" t="s">
         <v>371</v>
@@ -7312,14 +7316,16 @@
         <v>79</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8"/>
       <c r="F46" s="8" t="s">
-        <v>371</v>
-      </c>
-      <c r="G46" s="10"/>
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
     </row>
     <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A47" s="4" t="s">
@@ -7385,7 +7391,9 @@
       </c>
       <c r="D51" s="4"/>
       <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G51" s="9"/>
     </row>
     <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -7559,7 +7567,9 @@
       </c>
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G63" s="9"/>
     </row>
     <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -7706,7 +7716,9 @@
       </c>
       <c r="D72" s="8"/>
       <c r="E72" s="8"/>
-      <c r="F72" s="8"/>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G72" s="10"/>
     </row>
     <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -7768,7 +7780,9 @@
       </c>
       <c r="D76" s="8"/>
       <c r="E76" s="8"/>
-      <c r="F76" s="8"/>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G76" s="10"/>
     </row>
     <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -7884,7 +7898,9 @@
       </c>
       <c r="D84" s="8"/>
       <c r="E84" s="8"/>
-      <c r="F84" s="8"/>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G84" s="10"/>
     </row>
     <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
@@ -7953,7 +7969,9 @@
       <c r="E89" s="4" t="s">
         <v>345</v>
       </c>
-      <c r="F89" s="4"/>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G89" s="9"/>
     </row>
     <row r="90" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
@@ -8954,7 +8972,9 @@
       <c r="E154" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="F154" s="8"/>
+      <c r="F154" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G154" s="10"/>
     </row>
     <row r="155" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA MARÇO: CHECKLIST 16/03 15h
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C90CBD-B162-4F03-9C37-BC44CE7ECEA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE06A67-9170-4125-AC3C-72294E96C76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1339" uniqueCount="388">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1204,6 +1204,9 @@
   </si>
   <si>
     <t xml:space="preserve"> José Mecias Dos Santos /  86995749413</t>
+  </si>
+  <si>
+    <t>Leandro Ferreira de Souza / 86 8821-0081</t>
   </si>
 </sst>
 </file>
@@ -6989,7 +6992,9 @@
       <c r="C23" s="4" t="s">
         <v>383</v>
       </c>
-      <c r="D23" s="4"/>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
       <c r="E23" s="4" t="s">
         <v>386</v>
       </c>
@@ -7074,7 +7079,9 @@
       </c>
       <c r="D28" s="8"/>
       <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G28" s="10"/>
     </row>
     <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -8513,7 +8520,9 @@
       </c>
       <c r="D125" s="4"/>
       <c r="E125" s="4"/>
-      <c r="F125" s="4"/>
+      <c r="F125" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G125" s="9"/>
     </row>
     <row r="126" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA FROTA POTY: 17/03 16H
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE06A67-9170-4125-AC3C-72294E96C76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A653CC96-9C9B-433E-BC00-366766073444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
     <sheet name="13" sheetId="3" r:id="rId2"/>
     <sheet name="16" sheetId="4" r:id="rId3"/>
+    <sheet name="17" sheetId="5" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'13'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'16'!$A$6:$G$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'17'!$A$6:$G$170</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1339" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1938" uniqueCount="411">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1207,6 +1209,75 @@
   </si>
   <si>
     <t>Leandro Ferreira de Souza / 86 8821-0081</t>
+  </si>
+  <si>
+    <t>JACKSON</t>
+  </si>
+  <si>
+    <t>ADALTO</t>
+  </si>
+  <si>
+    <t>LEANDRO</t>
+  </si>
+  <si>
+    <t>LEONARDO</t>
+  </si>
+  <si>
+    <t>SAMUEL - TRANSPORTE UCP</t>
+  </si>
+  <si>
+    <t>JOSUE</t>
+  </si>
+  <si>
+    <t>EMANUEL</t>
+  </si>
+  <si>
+    <t>FRANK</t>
+  </si>
+  <si>
+    <t>ISRAEL</t>
+  </si>
+  <si>
+    <t>RONALDO</t>
+  </si>
+  <si>
+    <t>ANTONIO REIS</t>
+  </si>
+  <si>
+    <t>AGENI</t>
+  </si>
+  <si>
+    <t>GEOVANE</t>
+  </si>
+  <si>
+    <t>FRANCISCO CARDOSO</t>
+  </si>
+  <si>
+    <t>GUSTAVO</t>
+  </si>
+  <si>
+    <t>RAIMUNDO</t>
+  </si>
+  <si>
+    <t>JOAO COSTA</t>
+  </si>
+  <si>
+    <t>AMICIO</t>
+  </si>
+  <si>
+    <t>ALMEIDA / VALDIR</t>
+  </si>
+  <si>
+    <t>FRANCISCO</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERENCIA: 17/03/2026</t>
+  </si>
+  <si>
+    <t>PIRIPIRI</t>
+  </si>
+  <si>
+    <t>AGUA BRANCA</t>
   </si>
 </sst>
 </file>
@@ -1354,7 +1425,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1383,6 +1454,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1545,6 +1619,59 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65B41B34-48E6-4834-BFF0-ACA23D7EBE16}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D392C67-9860-4350-9ED5-445ED13666B4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1911,45 +2038,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="14" t="s">
         <v>338</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -4297,45 +4424,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -6677,45 +6804,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -7518,8 +7645,12 @@
         <v>104</v>
       </c>
       <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F59" s="4"/>
       <c r="G59" s="9"/>
     </row>
@@ -7917,39 +8048,57 @@
       <c r="B85" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C85" s="4"/>
-      <c r="D85" s="4"/>
-      <c r="E85" s="4"/>
+      <c r="C85" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F85" s="4"/>
       <c r="G85" s="9"/>
     </row>
-    <row r="86" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A86" s="8" t="s">
         <v>157</v>
       </c>
       <c r="B86" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="C86" s="8"/>
-      <c r="D86" s="8"/>
-      <c r="E86" s="8"/>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F86" s="8"/>
       <c r="G86" s="10"/>
     </row>
-    <row r="87" spans="1:7" s="7" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A87" s="4" t="s">
         <v>159</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="C87" s="4"/>
-      <c r="D87" s="4"/>
-      <c r="E87" s="4"/>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F87" s="4"/>
       <c r="G87" s="9"/>
     </row>
-    <row r="88" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A88" s="8" t="s">
         <v>161</v>
       </c>
@@ -7957,22 +8106,28 @@
         <v>162</v>
       </c>
       <c r="C88" s="8"/>
-      <c r="D88" s="8"/>
-      <c r="E88" s="8"/>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F88" s="8"/>
       <c r="G88" s="10"/>
     </row>
-    <row r="89" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A89" s="4" t="s">
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="12" t="s">
         <v>163</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="C89" s="4" t="s">
+      <c r="C89" s="12" t="s">
         <v>376</v>
       </c>
-      <c r="D89" s="4"/>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
       <c r="E89" s="4" t="s">
         <v>345</v>
       </c>
@@ -7981,46 +8136,64 @@
       </c>
       <c r="G89" s="9"/>
     </row>
-    <row r="90" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A90" s="8" t="s">
         <v>165</v>
       </c>
       <c r="B90" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="C90" s="8"/>
-      <c r="D90" s="8"/>
-      <c r="E90" s="8"/>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F90" s="8"/>
       <c r="G90" s="10"/>
     </row>
-    <row r="91" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A91" s="4" t="s">
         <v>167</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C91" s="4"/>
-      <c r="D91" s="4"/>
-      <c r="E91" s="4"/>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F91" s="4"/>
       <c r="G91" s="9"/>
     </row>
-    <row r="92" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A92" s="8" t="s">
         <v>169</v>
       </c>
       <c r="B92" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C92" s="8"/>
-      <c r="D92" s="8"/>
-      <c r="E92" s="8"/>
+      <c r="C92" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F92" s="8"/>
       <c r="G92" s="10"/>
     </row>
-    <row r="93" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A93" s="4" t="s">
         <v>171</v>
       </c>
@@ -8028,12 +8201,16 @@
         <v>172</v>
       </c>
       <c r="C93" s="4"/>
-      <c r="D93" s="4"/>
-      <c r="E93" s="4"/>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F93" s="4"/>
       <c r="G93" s="9"/>
     </row>
-    <row r="94" spans="1:7" s="7" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A94" s="8" t="s">
         <v>173</v>
       </c>
@@ -8046,7 +8223,7 @@
       <c r="F94" s="8"/>
       <c r="G94" s="10"/>
     </row>
-    <row r="95" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="4" t="s">
         <v>175</v>
       </c>
@@ -8059,7 +8236,7 @@
       <c r="F95" s="4"/>
       <c r="G95" s="9"/>
     </row>
-    <row r="96" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="8" t="s">
         <v>177</v>
       </c>
@@ -8072,7 +8249,7 @@
       <c r="F96" s="8"/>
       <c r="G96" s="10"/>
     </row>
-    <row r="97" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="4" t="s">
         <v>179</v>
       </c>
@@ -8093,7 +8270,7 @@
       </c>
       <c r="G97" s="9"/>
     </row>
-    <row r="98" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="8" t="s">
         <v>181</v>
       </c>
@@ -8108,7 +8285,7 @@
       <c r="F98" s="8"/>
       <c r="G98" s="10"/>
     </row>
-    <row r="99" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="4" t="s">
         <v>183</v>
       </c>
@@ -8121,7 +8298,7 @@
       <c r="F99" s="4"/>
       <c r="G99" s="9"/>
     </row>
-    <row r="100" spans="1:7" s="7" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="8" t="s">
         <v>185</v>
       </c>
@@ -8144,7 +8321,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="101" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="4" t="s">
         <v>187</v>
       </c>
@@ -8165,7 +8342,7 @@
       </c>
       <c r="G101" s="9"/>
     </row>
-    <row r="102" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="8" t="s">
         <v>189</v>
       </c>
@@ -8180,7 +8357,7 @@
       <c r="F102" s="8"/>
       <c r="G102" s="10"/>
     </row>
-    <row r="103" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="4" t="s">
         <v>191</v>
       </c>
@@ -8197,7 +8374,7 @@
       </c>
       <c r="G103" s="9"/>
     </row>
-    <row r="104" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="8" t="s">
         <v>193</v>
       </c>
@@ -8210,7 +8387,7 @@
       <c r="F104" s="8"/>
       <c r="G104" s="10"/>
     </row>
-    <row r="105" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="4" t="s">
         <v>195</v>
       </c>
@@ -8223,7 +8400,7 @@
       <c r="F105" s="4"/>
       <c r="G105" s="9"/>
     </row>
-    <row r="106" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="8" t="s">
         <v>197</v>
       </c>
@@ -8236,7 +8413,7 @@
       <c r="F106" s="8"/>
       <c r="G106" s="10"/>
     </row>
-    <row r="107" spans="1:7" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A107" s="4" t="s">
         <v>199</v>
       </c>
@@ -8257,7 +8434,7 @@
       </c>
       <c r="G107" s="9"/>
     </row>
-    <row r="108" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="8" t="s">
         <v>201</v>
       </c>
@@ -8276,7 +8453,7 @@
       </c>
       <c r="G108" s="10"/>
     </row>
-    <row r="109" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A109" s="4" t="s">
         <v>203</v>
       </c>
@@ -8299,7 +8476,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="110" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="8" t="s">
         <v>205</v>
       </c>
@@ -8316,7 +8493,7 @@
       </c>
       <c r="G110" s="10"/>
     </row>
-    <row r="111" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A111" s="4" t="s">
         <v>207</v>
       </c>
@@ -8331,7 +8508,7 @@
       <c r="F111" s="4"/>
       <c r="G111" s="9"/>
     </row>
-    <row r="112" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A112" s="8" t="s">
         <v>209</v>
       </c>
@@ -8344,7 +8521,7 @@
       <c r="F112" s="8"/>
       <c r="G112" s="10"/>
     </row>
-    <row r="113" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A113" s="4" t="s">
         <v>211</v>
       </c>
@@ -8365,7 +8542,7 @@
       </c>
       <c r="G113" s="9"/>
     </row>
-    <row r="114" spans="1:7" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A114" s="8" t="s">
         <v>213</v>
       </c>
@@ -8373,12 +8550,16 @@
         <v>214</v>
       </c>
       <c r="C114" s="8"/>
-      <c r="D114" s="8"/>
-      <c r="E114" s="8"/>
+      <c r="D114" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F114" s="8"/>
       <c r="G114" s="10"/>
     </row>
-    <row r="115" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A115" s="4" t="s">
         <v>215</v>
       </c>
@@ -8391,7 +8572,7 @@
       <c r="F115" s="4"/>
       <c r="G115" s="9"/>
     </row>
-    <row r="116" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="8" t="s">
         <v>217</v>
       </c>
@@ -8399,25 +8580,35 @@
         <v>218</v>
       </c>
       <c r="C116" s="8"/>
-      <c r="D116" s="8"/>
-      <c r="E116" s="8"/>
+      <c r="D116" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F116" s="8"/>
       <c r="G116" s="10"/>
     </row>
-    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="4" t="s">
         <v>219</v>
       </c>
       <c r="B117" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="C117" s="4"/>
-      <c r="D117" s="4"/>
-      <c r="E117" s="4"/>
+      <c r="C117" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D117" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E117" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F117" s="4"/>
       <c r="G117" s="9"/>
     </row>
-    <row r="118" spans="1:7" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="8" t="s">
         <v>221</v>
       </c>
@@ -8425,38 +8616,54 @@
         <v>222</v>
       </c>
       <c r="C118" s="8"/>
-      <c r="D118" s="8"/>
-      <c r="E118" s="8"/>
+      <c r="D118" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F118" s="8"/>
       <c r="G118" s="10"/>
     </row>
-    <row r="119" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="4" t="s">
         <v>223</v>
       </c>
       <c r="B119" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="C119" s="4"/>
-      <c r="D119" s="4"/>
-      <c r="E119" s="4"/>
+      <c r="C119" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D119" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E119" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F119" s="4"/>
       <c r="G119" s="9"/>
     </row>
-    <row r="120" spans="1:7" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="8" t="s">
         <v>225</v>
       </c>
       <c r="B120" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="C120" s="8"/>
-      <c r="D120" s="8"/>
-      <c r="E120" s="8"/>
+      <c r="C120" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D120" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F120" s="8"/>
       <c r="G120" s="10"/>
     </row>
-    <row r="121" spans="1:7" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="4" t="s">
         <v>227</v>
       </c>
@@ -8464,38 +8671,54 @@
         <v>228</v>
       </c>
       <c r="C121" s="4"/>
-      <c r="D121" s="4"/>
-      <c r="E121" s="4"/>
+      <c r="D121" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E121" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F121" s="4"/>
       <c r="G121" s="9"/>
     </row>
-    <row r="122" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="8" t="s">
         <v>229</v>
       </c>
       <c r="B122" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="C122" s="8"/>
-      <c r="D122" s="8"/>
-      <c r="E122" s="8"/>
+      <c r="C122" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E122" s="8" t="s">
+        <v>392</v>
+      </c>
       <c r="F122" s="8"/>
       <c r="G122" s="10"/>
     </row>
-    <row r="123" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A123" s="4" t="s">
         <v>231</v>
       </c>
       <c r="B123" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="C123" s="4"/>
-      <c r="D123" s="4"/>
-      <c r="E123" s="4"/>
+      <c r="C123" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E123" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F123" s="4"/>
       <c r="G123" s="9"/>
     </row>
-    <row r="124" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="8" t="s">
         <v>233</v>
       </c>
@@ -8508,7 +8731,7 @@
       <c r="F124" s="8"/>
       <c r="G124" s="10"/>
     </row>
-    <row r="125" spans="1:7" s="7" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="4" t="s">
         <v>235</v>
       </c>
@@ -8525,7 +8748,7 @@
       </c>
       <c r="G125" s="9"/>
     </row>
-    <row r="126" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="8" t="s">
         <v>237</v>
       </c>
@@ -8538,7 +8761,7 @@
       <c r="F126" s="8"/>
       <c r="G126" s="10"/>
     </row>
-    <row r="127" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="4" t="s">
         <v>239</v>
       </c>
@@ -8559,7 +8782,7 @@
       </c>
       <c r="G127" s="9"/>
     </row>
-    <row r="128" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="8" t="s">
         <v>241</v>
       </c>
@@ -8576,7 +8799,7 @@
       </c>
       <c r="G128" s="10"/>
     </row>
-    <row r="129" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="4" t="s">
         <v>243</v>
       </c>
@@ -8591,7 +8814,7 @@
       <c r="F129" s="4"/>
       <c r="G129" s="9"/>
     </row>
-    <row r="130" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="8" t="s">
         <v>245</v>
       </c>
@@ -8608,7 +8831,7 @@
       </c>
       <c r="G130" s="10"/>
     </row>
-    <row r="131" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="4" t="s">
         <v>247</v>
       </c>
@@ -8621,7 +8844,7 @@
       <c r="F131" s="4"/>
       <c r="G131" s="9"/>
     </row>
-    <row r="132" spans="1:7" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="8" t="s">
         <v>249</v>
       </c>
@@ -8644,7 +8867,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="133" spans="1:7" s="7" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="4" t="s">
         <v>251</v>
       </c>
@@ -8659,7 +8882,7 @@
       <c r="F133" s="4"/>
       <c r="G133" s="9"/>
     </row>
-    <row r="134" spans="1:7" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="8" t="s">
         <v>253</v>
       </c>
@@ -8680,7 +8903,7 @@
       </c>
       <c r="G134" s="10"/>
     </row>
-    <row r="135" spans="1:7" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="4" t="s">
         <v>255</v>
       </c>
@@ -8701,7 +8924,7 @@
       </c>
       <c r="G135" s="9"/>
     </row>
-    <row r="136" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A136" s="8" t="s">
         <v>257</v>
       </c>
@@ -8716,7 +8939,7 @@
       <c r="F136" s="8"/>
       <c r="G136" s="10"/>
     </row>
-    <row r="137" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A137" s="4" t="s">
         <v>259</v>
       </c>
@@ -8737,7 +8960,7 @@
       </c>
       <c r="G137" s="9"/>
     </row>
-    <row r="138" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A138" s="8" t="s">
         <v>261</v>
       </c>
@@ -8758,7 +8981,7 @@
       </c>
       <c r="G138" s="10"/>
     </row>
-    <row r="139" spans="1:7" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A139" s="4" t="s">
         <v>263</v>
       </c>
@@ -8779,7 +9002,7 @@
       </c>
       <c r="G139" s="9"/>
     </row>
-    <row r="140" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A140" s="8" t="s">
         <v>265</v>
       </c>
@@ -8792,7 +9015,7 @@
       <c r="F140" s="8"/>
       <c r="G140" s="10"/>
     </row>
-    <row r="141" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A141" s="4" t="s">
         <v>267</v>
       </c>
@@ -8805,7 +9028,7 @@
       <c r="F141" s="4"/>
       <c r="G141" s="9"/>
     </row>
-    <row r="142" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="8" t="s">
         <v>269</v>
       </c>
@@ -8822,7 +9045,7 @@
       </c>
       <c r="G142" s="10"/>
     </row>
-    <row r="143" spans="1:7" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A143" s="4" t="s">
         <v>271</v>
       </c>
@@ -8835,7 +9058,7 @@
       <c r="F143" s="4"/>
       <c r="G143" s="9"/>
     </row>
-    <row r="144" spans="1:7" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A144" s="8" t="s">
         <v>273</v>
       </c>
@@ -8852,7 +9075,7 @@
       </c>
       <c r="G144" s="10"/>
     </row>
-    <row r="145" spans="1:7" s="7" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A145" s="4" t="s">
         <v>275</v>
       </c>
@@ -8865,7 +9088,7 @@
       <c r="F145" s="4"/>
       <c r="G145" s="9"/>
     </row>
-    <row r="146" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A146" s="8" t="s">
         <v>277</v>
       </c>
@@ -8878,7 +9101,7 @@
       <c r="F146" s="8"/>
       <c r="G146" s="10"/>
     </row>
-    <row r="147" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A147" s="4" t="s">
         <v>279</v>
       </c>
@@ -8889,7 +9112,7 @@
       <c r="F147" s="4"/>
       <c r="G147" s="9"/>
     </row>
-    <row r="148" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A148" s="8" t="s">
         <v>281</v>
       </c>
@@ -8902,7 +9125,7 @@
       <c r="F148" s="8"/>
       <c r="G148" s="10"/>
     </row>
-    <row r="149" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A149" s="4" t="s">
         <v>283</v>
       </c>
@@ -8915,7 +9138,7 @@
       <c r="F149" s="4"/>
       <c r="G149" s="9"/>
     </row>
-    <row r="150" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A150" s="8" t="s">
         <v>285</v>
       </c>
@@ -8928,7 +9151,7 @@
       <c r="F150" s="8"/>
       <c r="G150" s="10"/>
     </row>
-    <row r="151" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A151" s="4" t="s">
         <v>287</v>
       </c>
@@ -8941,7 +9164,7 @@
       <c r="F151" s="4"/>
       <c r="G151" s="9"/>
     </row>
-    <row r="152" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A152" s="8" t="s">
         <v>289</v>
       </c>
@@ -8954,7 +9177,7 @@
       <c r="F152" s="8"/>
       <c r="G152" s="10"/>
     </row>
-    <row r="153" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A153" s="4" t="s">
         <v>291</v>
       </c>
@@ -8967,7 +9190,7 @@
       <c r="F153" s="4"/>
       <c r="G153" s="9"/>
     </row>
-    <row r="154" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A154" s="8" t="s">
         <v>293</v>
       </c>
@@ -8986,7 +9209,7 @@
       </c>
       <c r="G154" s="10"/>
     </row>
-    <row r="155" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A155" s="4" t="s">
         <v>295</v>
       </c>
@@ -8999,7 +9222,7 @@
       <c r="F155" s="4"/>
       <c r="G155" s="9"/>
     </row>
-    <row r="156" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A156" s="8" t="s">
         <v>297</v>
       </c>
@@ -9012,7 +9235,7 @@
       <c r="F156" s="8"/>
       <c r="G156" s="10"/>
     </row>
-    <row r="157" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A157" s="4" t="s">
         <v>299</v>
       </c>
@@ -9025,7 +9248,7 @@
       <c r="F157" s="4"/>
       <c r="G157" s="9"/>
     </row>
-    <row r="158" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A158" s="8" t="s">
         <v>301</v>
       </c>
@@ -9038,7 +9261,7 @@
       <c r="F158" s="8"/>
       <c r="G158" s="10"/>
     </row>
-    <row r="159" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A159" s="4" t="s">
         <v>303</v>
       </c>
@@ -9051,7 +9274,7 @@
       <c r="F159" s="4"/>
       <c r="G159" s="9"/>
     </row>
-    <row r="160" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A160" s="8" t="s">
         <v>305</v>
       </c>
@@ -9064,7 +9287,7 @@
       <c r="F160" s="8"/>
       <c r="G160" s="10"/>
     </row>
-    <row r="161" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A161" s="4" t="s">
         <v>307</v>
       </c>
@@ -9077,7 +9300,7 @@
       <c r="F161" s="4"/>
       <c r="G161" s="9"/>
     </row>
-    <row r="162" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A162" s="8" t="s">
         <v>309</v>
       </c>
@@ -9090,7 +9313,7 @@
       <c r="F162" s="8"/>
       <c r="G162" s="10"/>
     </row>
-    <row r="163" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A163" s="4" t="s">
         <v>311</v>
       </c>
@@ -9103,7 +9326,7 @@
       <c r="F163" s="4"/>
       <c r="G163" s="9"/>
     </row>
-    <row r="164" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A164" s="8" t="s">
         <v>313</v>
       </c>
@@ -9116,7 +9339,7 @@
       <c r="F164" s="8"/>
       <c r="G164" s="10"/>
     </row>
-    <row r="165" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A165" s="4" t="s">
         <v>315</v>
       </c>
@@ -9129,7 +9352,7 @@
       <c r="F165" s="4"/>
       <c r="G165" s="9"/>
     </row>
-    <row r="166" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A166" s="8" t="s">
         <v>317</v>
       </c>
@@ -9142,7 +9365,7 @@
       <c r="F166" s="8"/>
       <c r="G166" s="10"/>
     </row>
-    <row r="167" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A167" s="4" t="s">
         <v>319</v>
       </c>
@@ -9163,7 +9386,7 @@
       </c>
       <c r="G167" s="9"/>
     </row>
-    <row r="168" spans="1:7" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A168" s="8" t="s">
         <v>321</v>
       </c>
@@ -9176,7 +9399,7 @@
       <c r="F168" s="8"/>
       <c r="G168" s="10"/>
     </row>
-    <row r="169" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A169" s="4" t="s">
         <v>323</v>
       </c>
@@ -9189,7 +9412,2657 @@
       <c r="F169" s="4"/>
       <c r="G169" s="9"/>
     </row>
-    <row r="170" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="170" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A170" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B170" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C170" s="8"/>
+      <c r="D170" s="8"/>
+      <c r="E170" s="8"/>
+      <c r="F170" s="8"/>
+      <c r="G170" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G170" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E52299B-11B1-4F1E-B7ED-5D1B0F49AF8F}">
+  <dimension ref="A1:G170"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="39.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="38.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="10"/>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="10"/>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="8"/>
+      <c r="G56" s="10"/>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="10"/>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F59" s="4"/>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="10"/>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8"/>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10"/>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="9"/>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8"/>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4"/>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8"/>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="8"/>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10"/>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8"/>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8"/>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F85" s="4"/>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F86" s="8"/>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F87" s="4"/>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8"/>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F88" s="8"/>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F90" s="8"/>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F91" s="4"/>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F92" s="8"/>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F93" s="4"/>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8"/>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8"/>
+      <c r="F94" s="8"/>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+      <c r="F95" s="4"/>
+      <c r="G95" s="9"/>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="8"/>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8"/>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8"/>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+      <c r="F105" s="4"/>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8"/>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8"/>
+      <c r="F106" s="8"/>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8"/>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8"/>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="C112" s="8"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="8"/>
+      <c r="G112" s="10"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E113" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="9"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C114" s="8"/>
+      <c r="D114" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F114" s="8"/>
+      <c r="G114" s="10"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C115" s="4"/>
+      <c r="D115" s="4"/>
+      <c r="E115" s="4"/>
+      <c r="F115" s="4"/>
+      <c r="G115" s="9"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C116" s="8"/>
+      <c r="D116" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F116" s="8"/>
+      <c r="G116" s="10"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D117" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E117" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F117" s="4"/>
+      <c r="G117" s="9"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B118" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C118" s="8"/>
+      <c r="D118" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F118" s="8"/>
+      <c r="G118" s="10"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D119" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E119" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F119" s="4"/>
+      <c r="G119" s="9"/>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C120" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D120" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F120" s="8"/>
+      <c r="G120" s="10"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C121" s="4"/>
+      <c r="D121" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E121" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F121" s="4"/>
+      <c r="G121" s="9"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B122" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C122" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E122" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F122" s="8"/>
+      <c r="G122" s="10"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E123" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F123" s="4"/>
+      <c r="G123" s="9"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B124" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C124" s="8"/>
+      <c r="D124" s="8"/>
+      <c r="E124" s="8"/>
+      <c r="F124" s="8"/>
+      <c r="G124" s="10"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="D125" s="4"/>
+      <c r="E125" s="4"/>
+      <c r="F125" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G125" s="9"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C126" s="8"/>
+      <c r="D126" s="8"/>
+      <c r="E126" s="8"/>
+      <c r="F126" s="8"/>
+      <c r="G126" s="10"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E127" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G127" s="9"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C128" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="8"/>
+      <c r="E128" s="8"/>
+      <c r="F128" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G128" s="10"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="4"/>
+      <c r="E129" s="4"/>
+      <c r="F129" s="4"/>
+      <c r="G129" s="9"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="8"/>
+      <c r="E130" s="8"/>
+      <c r="F130" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G130" s="10"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C131" s="4"/>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+      <c r="G131" s="9"/>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D132" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F132" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D133" s="4"/>
+      <c r="E133" s="4"/>
+      <c r="F133" s="4"/>
+      <c r="G133" s="9"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C134" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D134" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F134" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="10"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E135" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G135" s="9"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C136" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D136" s="8"/>
+      <c r="E136" s="8"/>
+      <c r="F136" s="8"/>
+      <c r="G136" s="10"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E137" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="9"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C138" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D138" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F138" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="10"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D139" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E139" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G139" s="9"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C140" s="8"/>
+      <c r="D140" s="8"/>
+      <c r="E140" s="8"/>
+      <c r="F140" s="8"/>
+      <c r="G140" s="10"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C141" s="4"/>
+      <c r="D141" s="4"/>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="9"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C142" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="8"/>
+      <c r="E142" s="8"/>
+      <c r="F142" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G142" s="10"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4"/>
+      <c r="G143" s="9"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="8"/>
+      <c r="E144" s="8"/>
+      <c r="F144" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G144" s="10"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C145" s="4"/>
+      <c r="D145" s="4"/>
+      <c r="E145" s="4"/>
+      <c r="F145" s="4"/>
+      <c r="G145" s="9"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B146" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C146" s="8"/>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8"/>
+      <c r="G146" s="10"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="E147" s="4"/>
+      <c r="F147" s="4"/>
+      <c r="G147" s="9"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B148" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C148" s="8"/>
+      <c r="D148" s="8"/>
+      <c r="E148" s="8"/>
+      <c r="F148" s="8"/>
+      <c r="G148" s="10"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C149" s="4"/>
+      <c r="D149" s="4"/>
+      <c r="E149" s="4"/>
+      <c r="F149" s="4"/>
+      <c r="G149" s="9"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C150" s="8"/>
+      <c r="D150" s="8"/>
+      <c r="E150" s="8"/>
+      <c r="F150" s="8"/>
+      <c r="G150" s="10"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="9"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B152" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C152" s="8"/>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
+      <c r="F152" s="8"/>
+      <c r="G152" s="10"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C153" s="4"/>
+      <c r="D153" s="4"/>
+      <c r="E153" s="4"/>
+      <c r="F153" s="4"/>
+      <c r="G153" s="9"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C154" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="D154" s="8"/>
+      <c r="E154" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F154" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="10"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4"/>
+      <c r="G155" s="9"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C156" s="8"/>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8"/>
+      <c r="F156" s="8"/>
+      <c r="G156" s="10"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C157" s="4"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4"/>
+      <c r="G157" s="9"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B158" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C158" s="8"/>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8"/>
+      <c r="F158" s="8"/>
+      <c r="G158" s="10"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="9"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B160" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C160" s="8"/>
+      <c r="D160" s="8"/>
+      <c r="E160" s="8"/>
+      <c r="F160" s="8"/>
+      <c r="G160" s="10"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+      <c r="G161" s="9"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B162" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C162" s="8"/>
+      <c r="D162" s="8"/>
+      <c r="E162" s="8"/>
+      <c r="F162" s="8"/>
+      <c r="G162" s="10"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+      <c r="G163" s="9"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B164" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C164" s="8"/>
+      <c r="D164" s="8"/>
+      <c r="E164" s="8"/>
+      <c r="F164" s="8"/>
+      <c r="G164" s="10"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C165" s="4"/>
+      <c r="D165" s="4"/>
+      <c r="E165" s="4"/>
+      <c r="F165" s="4"/>
+      <c r="G165" s="9"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B166" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C166" s="8"/>
+      <c r="D166" s="8"/>
+      <c r="E166" s="8"/>
+      <c r="F166" s="8"/>
+      <c r="G166" s="10"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D167" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E167" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G167" s="9"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B168" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C168" s="8"/>
+      <c r="D168" s="8"/>
+      <c r="E168" s="8"/>
+      <c r="F168" s="8"/>
+      <c r="G168" s="10"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C169" s="4"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="9"/>
+    </row>
+    <row r="170" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A170" s="8" t="s">
         <v>325</v>
       </c>

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA FROTA POTY: 18/03 8:25H
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,21 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A653CC96-9C9B-433E-BC00-366766073444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6872EE94-3E42-455C-BE91-56306C1ED632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
     <sheet name="13" sheetId="3" r:id="rId2"/>
     <sheet name="16" sheetId="4" r:id="rId3"/>
     <sheet name="17" sheetId="5" r:id="rId4"/>
+    <sheet name="18" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'13'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'16'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'17'!$A$6:$G$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'18'!$A$6:$G$170</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1938" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2489" uniqueCount="414">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1278,6 +1280,15 @@
   </si>
   <si>
     <t>AGUA BRANCA</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERENCIA: 18/03/2026</t>
+  </si>
+  <si>
+    <t>SANTA RITA DO PIAUI</t>
+  </si>
+  <si>
+    <t>SÃO MIGUEL DO TAPUIO</t>
   </si>
 </sst>
 </file>
@@ -1704,6 +1715,59 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9124FB0A-15F8-4690-8959-A8A7D953F144}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -12084,4 +12148,2654 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{255AD8CD-DB98-4F1E-AEC5-D12CAEE762DC}">
+  <dimension ref="A1:G170"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="39.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="38.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
+        <v>411</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="10"/>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="10"/>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="8"/>
+      <c r="G56" s="10"/>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="10"/>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F59" s="4"/>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="10"/>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8"/>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10"/>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="9"/>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8"/>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4"/>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8"/>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="8"/>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10"/>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8"/>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8"/>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F85" s="4"/>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F86" s="8"/>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F87" s="4"/>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8"/>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F88" s="8"/>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F90" s="8"/>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F91" s="4"/>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F92" s="8"/>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F93" s="4"/>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8"/>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8"/>
+      <c r="F94" s="8"/>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+      <c r="F95" s="4"/>
+      <c r="G95" s="9"/>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="8"/>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8"/>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8"/>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+      <c r="F105" s="4"/>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8"/>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8"/>
+      <c r="F106" s="8"/>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8"/>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8"/>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="C112" s="8"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="8"/>
+      <c r="G112" s="10"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E113" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="9"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C114" s="8"/>
+      <c r="D114" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F114" s="8"/>
+      <c r="G114" s="10"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C115" s="4"/>
+      <c r="D115" s="4"/>
+      <c r="E115" s="4"/>
+      <c r="F115" s="4"/>
+      <c r="G115" s="9"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C116" s="8"/>
+      <c r="D116" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F116" s="8"/>
+      <c r="G116" s="10"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D117" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E117" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F117" s="4"/>
+      <c r="G117" s="9"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B118" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C118" s="8"/>
+      <c r="D118" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F118" s="8"/>
+      <c r="G118" s="10"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D119" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E119" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F119" s="4"/>
+      <c r="G119" s="9"/>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C120" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D120" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F120" s="8"/>
+      <c r="G120" s="10"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C121" s="4"/>
+      <c r="D121" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E121" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F121" s="4"/>
+      <c r="G121" s="9"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B122" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C122" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E122" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F122" s="8"/>
+      <c r="G122" s="10"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E123" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F123" s="4"/>
+      <c r="G123" s="9"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B124" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C124" s="8"/>
+      <c r="D124" s="8"/>
+      <c r="E124" s="8"/>
+      <c r="F124" s="8"/>
+      <c r="G124" s="10"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D125" s="4"/>
+      <c r="E125" s="4"/>
+      <c r="F125" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G125" s="9"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C126" s="8"/>
+      <c r="D126" s="8"/>
+      <c r="E126" s="8"/>
+      <c r="F126" s="8"/>
+      <c r="G126" s="10"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E127" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G127" s="9"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C128" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="8"/>
+      <c r="E128" s="8"/>
+      <c r="F128" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G128" s="10"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="4"/>
+      <c r="E129" s="4"/>
+      <c r="F129" s="4"/>
+      <c r="G129" s="9"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="8"/>
+      <c r="E130" s="8"/>
+      <c r="F130" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G130" s="10"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C131" s="4"/>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+      <c r="G131" s="9"/>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D132" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F132" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D133" s="4"/>
+      <c r="E133" s="4"/>
+      <c r="F133" s="4"/>
+      <c r="G133" s="9"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C134" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D134" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F134" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="10"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E135" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G135" s="9"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C136" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D136" s="8"/>
+      <c r="E136" s="8"/>
+      <c r="F136" s="8"/>
+      <c r="G136" s="10"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E137" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="9"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C138" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D138" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F138" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="10"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D139" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E139" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G139" s="9"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C140" s="8"/>
+      <c r="D140" s="8"/>
+      <c r="E140" s="8"/>
+      <c r="F140" s="8"/>
+      <c r="G140" s="10"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C141" s="4"/>
+      <c r="D141" s="4"/>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="9"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C142" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="8"/>
+      <c r="E142" s="8"/>
+      <c r="F142" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G142" s="10"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4"/>
+      <c r="G143" s="9"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="8"/>
+      <c r="E144" s="8"/>
+      <c r="F144" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G144" s="10"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C145" s="4"/>
+      <c r="D145" s="4"/>
+      <c r="E145" s="4"/>
+      <c r="F145" s="4"/>
+      <c r="G145" s="9"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B146" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C146" s="8"/>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8"/>
+      <c r="G146" s="10"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="E147" s="4"/>
+      <c r="F147" s="4"/>
+      <c r="G147" s="9"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B148" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C148" s="8"/>
+      <c r="D148" s="8"/>
+      <c r="E148" s="8"/>
+      <c r="F148" s="8"/>
+      <c r="G148" s="10"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C149" s="4"/>
+      <c r="D149" s="4"/>
+      <c r="E149" s="4"/>
+      <c r="F149" s="4"/>
+      <c r="G149" s="9"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C150" s="8"/>
+      <c r="D150" s="8"/>
+      <c r="E150" s="8"/>
+      <c r="F150" s="8"/>
+      <c r="G150" s="10"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="9"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B152" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C152" s="8"/>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
+      <c r="F152" s="8"/>
+      <c r="G152" s="10"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C153" s="4"/>
+      <c r="D153" s="4"/>
+      <c r="E153" s="4"/>
+      <c r="F153" s="4"/>
+      <c r="G153" s="9"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C154" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D154" s="8"/>
+      <c r="E154" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F154" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="10"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4"/>
+      <c r="G155" s="9"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C156" s="8"/>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8"/>
+      <c r="F156" s="8"/>
+      <c r="G156" s="10"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C157" s="4"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4"/>
+      <c r="G157" s="9"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B158" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C158" s="8"/>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8"/>
+      <c r="F158" s="8"/>
+      <c r="G158" s="10"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="9"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B160" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C160" s="8"/>
+      <c r="D160" s="8"/>
+      <c r="E160" s="8"/>
+      <c r="F160" s="8"/>
+      <c r="G160" s="10"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+      <c r="G161" s="9"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B162" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C162" s="8"/>
+      <c r="D162" s="8"/>
+      <c r="E162" s="8"/>
+      <c r="F162" s="8"/>
+      <c r="G162" s="10"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+      <c r="G163" s="9"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B164" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C164" s="8"/>
+      <c r="D164" s="8"/>
+      <c r="E164" s="8"/>
+      <c r="F164" s="8"/>
+      <c r="G164" s="10"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C165" s="4"/>
+      <c r="D165" s="4"/>
+      <c r="E165" s="4"/>
+      <c r="F165" s="4"/>
+      <c r="G165" s="9"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B166" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C166" s="8"/>
+      <c r="D166" s="8"/>
+      <c r="E166" s="8"/>
+      <c r="F166" s="8"/>
+      <c r="G166" s="10"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D167" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E167" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G167" s="9"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B168" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C168" s="8"/>
+      <c r="D168" s="8"/>
+      <c r="E168" s="8"/>
+      <c r="F168" s="8"/>
+      <c r="G168" s="10"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C169" s="4"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="9"/>
+    </row>
+    <row r="170" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A170" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B170" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C170" s="8"/>
+      <c r="D170" s="8"/>
+      <c r="E170" s="8"/>
+      <c r="F170" s="8"/>
+      <c r="G170" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G170" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA MARÇO: CHECKLIST 18/03 13h
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6872EE94-3E42-455C-BE91-56306C1ED632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{770C2C18-0A3E-483C-960C-9610F07EE1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2489" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2492" uniqueCount="415">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1289,6 +1289,9 @@
   </si>
   <si>
     <t>SÃO MIGUEL DO TAPUIO</t>
+  </si>
+  <si>
+    <t>Felipe Hudsom</t>
   </si>
 </sst>
 </file>
@@ -12564,10 +12567,14 @@
         <v>43</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>374</v>
-      </c>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>386</v>
+      </c>
       <c r="F28" s="8" t="s">
         <v>333</v>
       </c>
@@ -13851,7 +13858,9 @@
         <v>413</v>
       </c>
       <c r="D110" s="8"/>
-      <c r="E110" s="8"/>
+      <c r="E110" s="8" t="s">
+        <v>386</v>
+      </c>
       <c r="F110" s="8" t="s">
         <v>371</v>
       </c>
@@ -14795,7 +14804,8 @@
     <mergeCell ref="A1:G3"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
FECHAMENTO FEVEREIRO: ATIVOS INCIO 1 E 2 LANÇADOS:18/03 17H
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{770C2C18-0A3E-483C-960C-9610F07EE1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1CBC884-F719-468D-9621-0DBF325BE318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2492" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2495" uniqueCount="415">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -13198,17 +13198,21 @@
       </c>
       <c r="G70" s="10"/>
     </row>
-    <row r="71" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="4" t="s">
         <v>127</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="C71" s="4"/>
+      <c r="C71" s="4" t="s">
+        <v>377</v>
+      </c>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
-      <c r="F71" s="4"/>
+      <c r="F71" s="4" t="s">
+        <v>371</v>
+      </c>
       <c r="G71" s="9"/>
     </row>
     <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -13302,7 +13306,9 @@
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
-      <c r="F77" s="4"/>
+      <c r="F77" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G77" s="9"/>
     </row>
     <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA FROTA POTY: 19/03 8:08H
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1CBC884-F719-468D-9621-0DBF325BE318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C71F5B9-01A1-453D-8261-D0013660BF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="16" sheetId="4" r:id="rId3"/>
     <sheet name="17" sheetId="5" r:id="rId4"/>
     <sheet name="18" sheetId="6" r:id="rId5"/>
+    <sheet name="19" sheetId="7" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
@@ -25,6 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'16'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'17'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'18'!$A$6:$G$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'19'!$A$6:$G$170</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2495" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3056" uniqueCount="417">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1292,6 +1294,12 @@
   </si>
   <si>
     <t>Felipe Hudsom</t>
+  </si>
+  <si>
+    <t>ANTONIO ALMEIDA</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERENCIA: 19/03/2026</t>
   </si>
 </sst>
 </file>
@@ -1439,7 +1447,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1478,6 +1486,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1739,6 +1750,59 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9124FB0A-15F8-4690-8959-A8A7D953F144}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D46519E0-8A5D-41CE-9640-961A613AA8FF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -12155,14 +12219,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{255AD8CD-DB98-4F1E-AEC5-D12CAEE762DC}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G170"/>
   <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="5"/>
     <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
-    <col min="4" max="4" width="39.5703125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="38.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="5" customWidth="1"/>
     <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21" style="6" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="5"/>
@@ -12232,7 +12297,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A7" s="4" t="s">
         <v>0</v>
       </c>
@@ -12249,7 +12314,7 @@
       </c>
       <c r="G7" s="9"/>
     </row>
-    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A8" s="8" t="s">
         <v>2</v>
       </c>
@@ -12264,7 +12329,7 @@
       <c r="F8" s="8"/>
       <c r="G8" s="10"/>
     </row>
-    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A9" s="4" t="s">
         <v>4</v>
       </c>
@@ -12281,7 +12346,7 @@
       </c>
       <c r="G9" s="9"/>
     </row>
-    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A10" s="8" t="s">
         <v>6</v>
       </c>
@@ -12294,7 +12359,7 @@
       <c r="F10" s="8"/>
       <c r="G10" s="10"/>
     </row>
-    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
@@ -12311,7 +12376,7 @@
       </c>
       <c r="G11" s="9"/>
     </row>
-    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A12" s="8" t="s">
         <v>10</v>
       </c>
@@ -12324,7 +12389,7 @@
       <c r="F12" s="8"/>
       <c r="G12" s="10"/>
     </row>
-    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
@@ -12341,7 +12406,7 @@
       </c>
       <c r="G13" s="9"/>
     </row>
-    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A14" s="8" t="s">
         <v>14</v>
       </c>
@@ -12358,7 +12423,7 @@
       </c>
       <c r="G14" s="10"/>
     </row>
-    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
@@ -12375,7 +12440,7 @@
       </c>
       <c r="G15" s="9"/>
     </row>
-    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A16" s="8" t="s">
         <v>18</v>
       </c>
@@ -12390,7 +12455,7 @@
       <c r="F16" s="8"/>
       <c r="G16" s="10"/>
     </row>
-    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
@@ -12403,7 +12468,7 @@
       <c r="F17" s="4"/>
       <c r="G17" s="9"/>
     </row>
-    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
@@ -12416,7 +12481,7 @@
       <c r="F18" s="8"/>
       <c r="G18" s="10"/>
     </row>
-    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A19" s="4" t="s">
         <v>24</v>
       </c>
@@ -12429,7 +12494,7 @@
       <c r="F19" s="4"/>
       <c r="G19" s="9"/>
     </row>
-    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A20" s="8" t="s">
         <v>26</v>
       </c>
@@ -12442,7 +12507,7 @@
       <c r="F20" s="8"/>
       <c r="G20" s="10"/>
     </row>
-    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A21" s="4" t="s">
         <v>28</v>
       </c>
@@ -12457,7 +12522,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="9"/>
     </row>
-    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A22" s="8" t="s">
         <v>30</v>
       </c>
@@ -12474,7 +12539,7 @@
       </c>
       <c r="G22" s="10"/>
     </row>
-    <row r="23" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A23" s="4" t="s">
         <v>32</v>
       </c>
@@ -12495,7 +12560,7 @@
       </c>
       <c r="G23" s="9"/>
     </row>
-    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A24" s="8" t="s">
         <v>34</v>
       </c>
@@ -12508,7 +12573,7 @@
       <c r="F24" s="8"/>
       <c r="G24" s="10"/>
     </row>
-    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A25" s="4" t="s">
         <v>36</v>
       </c>
@@ -12525,7 +12590,7 @@
       </c>
       <c r="G25" s="9"/>
     </row>
-    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A26" s="8" t="s">
         <v>38</v>
       </c>
@@ -12542,7 +12607,7 @@
       </c>
       <c r="G26" s="10"/>
     </row>
-    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A27" s="4" t="s">
         <v>40</v>
       </c>
@@ -12559,7 +12624,7 @@
       </c>
       <c r="G27" s="9"/>
     </row>
-    <row r="28" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A28" s="8" t="s">
         <v>42</v>
       </c>
@@ -12580,7 +12645,7 @@
       </c>
       <c r="G28" s="10"/>
     </row>
-    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A29" s="4" t="s">
         <v>44</v>
       </c>
@@ -12593,7 +12658,7 @@
       <c r="F29" s="4"/>
       <c r="G29" s="9"/>
     </row>
-    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A30" s="8" t="s">
         <v>46</v>
       </c>
@@ -12606,7 +12671,7 @@
       <c r="F30" s="8"/>
       <c r="G30" s="10"/>
     </row>
-    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="4" t="s">
         <v>48</v>
       </c>
@@ -12619,7 +12684,7 @@
       <c r="F31" s="4"/>
       <c r="G31" s="9"/>
     </row>
-    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A32" s="8" t="s">
         <v>50</v>
       </c>
@@ -12632,7 +12697,7 @@
       <c r="F32" s="8"/>
       <c r="G32" s="10"/>
     </row>
-    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A33" s="4" t="s">
         <v>52</v>
       </c>
@@ -12645,7 +12710,7 @@
       <c r="F33" s="4"/>
       <c r="G33" s="9"/>
     </row>
-    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A34" s="8" t="s">
         <v>54</v>
       </c>
@@ -12658,7 +12723,7 @@
       <c r="F34" s="8"/>
       <c r="G34" s="10"/>
     </row>
-    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="4" t="s">
         <v>56</v>
       </c>
@@ -12681,7 +12746,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A36" s="8" t="s">
         <v>58</v>
       </c>
@@ -12694,7 +12759,7 @@
       <c r="F36" s="8"/>
       <c r="G36" s="10"/>
     </row>
-    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A37" s="4" t="s">
         <v>60</v>
       </c>
@@ -12707,7 +12772,7 @@
       <c r="F37" s="4"/>
       <c r="G37" s="9"/>
     </row>
-    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A38" s="8" t="s">
         <v>62</v>
       </c>
@@ -12720,7 +12785,7 @@
       <c r="F38" s="8"/>
       <c r="G38" s="10"/>
     </row>
-    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A39" s="4" t="s">
         <v>64</v>
       </c>
@@ -12733,7 +12798,7 @@
       <c r="F39" s="4"/>
       <c r="G39" s="9"/>
     </row>
-    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A40" s="8" t="s">
         <v>66</v>
       </c>
@@ -12746,7 +12811,7 @@
       <c r="F40" s="8"/>
       <c r="G40" s="10"/>
     </row>
-    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A41" s="4" t="s">
         <v>68</v>
       </c>
@@ -12759,7 +12824,7 @@
       <c r="F41" s="4"/>
       <c r="G41" s="9"/>
     </row>
-    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A42" s="8" t="s">
         <v>70</v>
       </c>
@@ -12772,7 +12837,7 @@
       <c r="F42" s="8"/>
       <c r="G42" s="10"/>
     </row>
-    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A43" s="4" t="s">
         <v>72</v>
       </c>
@@ -12785,7 +12850,7 @@
       <c r="F43" s="4"/>
       <c r="G43" s="9"/>
     </row>
-    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A44" s="8" t="s">
         <v>74</v>
       </c>
@@ -12798,7 +12863,7 @@
       <c r="F44" s="8"/>
       <c r="G44" s="10"/>
     </row>
-    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A45" s="4" t="s">
         <v>76</v>
       </c>
@@ -12811,7 +12876,7 @@
       <c r="F45" s="4"/>
       <c r="G45" s="9"/>
     </row>
-    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A46" s="8" t="s">
         <v>78</v>
       </c>
@@ -12830,7 +12895,7 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A47" s="4" t="s">
         <v>80</v>
       </c>
@@ -12843,7 +12908,7 @@
       <c r="F47" s="4"/>
       <c r="G47" s="9"/>
     </row>
-    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A48" s="8" t="s">
         <v>82</v>
       </c>
@@ -12856,7 +12921,7 @@
       <c r="F48" s="8"/>
       <c r="G48" s="10"/>
     </row>
-    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A49" s="4" t="s">
         <v>84</v>
       </c>
@@ -12869,7 +12934,7 @@
       <c r="F49" s="4"/>
       <c r="G49" s="9"/>
     </row>
-    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A50" s="8" t="s">
         <v>86</v>
       </c>
@@ -12882,7 +12947,7 @@
       <c r="F50" s="8"/>
       <c r="G50" s="10"/>
     </row>
-    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" hidden="1" x14ac:dyDescent="0.15">
       <c r="A51" s="4" t="s">
         <v>88</v>
       </c>
@@ -12899,7 +12964,7 @@
       </c>
       <c r="G51" s="9"/>
     </row>
-    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A52" s="8" t="s">
         <v>90</v>
       </c>
@@ -13017,13 +13082,11 @@
       <c r="D59" s="4" t="s">
         <v>405</v>
       </c>
-      <c r="E59" s="4" t="s">
-        <v>392</v>
-      </c>
+      <c r="E59" s="4"/>
       <c r="F59" s="4"/>
       <c r="G59" s="9"/>
     </row>
-    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A60" s="8" t="s">
         <v>105</v>
       </c>
@@ -13036,7 +13099,7 @@
       <c r="F60" s="8"/>
       <c r="G60" s="10"/>
     </row>
-    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A61" s="4" t="s">
         <v>107</v>
       </c>
@@ -13049,7 +13112,7 @@
       <c r="F61" s="4"/>
       <c r="G61" s="9"/>
     </row>
-    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A62" s="8" t="s">
         <v>109</v>
       </c>
@@ -13062,7 +13125,7 @@
       <c r="F62" s="8"/>
       <c r="G62" s="10"/>
     </row>
-    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A63" s="4" t="s">
         <v>111</v>
       </c>
@@ -13079,7 +13142,7 @@
       </c>
       <c r="G63" s="9"/>
     </row>
-    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A64" s="8" t="s">
         <v>113</v>
       </c>
@@ -13096,7 +13159,7 @@
       </c>
       <c r="G64" s="10"/>
     </row>
-    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A65" s="4" t="s">
         <v>115</v>
       </c>
@@ -13113,7 +13176,7 @@
       </c>
       <c r="G65" s="9"/>
     </row>
-    <row r="66" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A66" s="8" t="s">
         <v>117</v>
       </c>
@@ -13134,7 +13197,7 @@
       </c>
       <c r="G66" s="10"/>
     </row>
-    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A67" s="4" t="s">
         <v>119</v>
       </c>
@@ -13147,7 +13210,7 @@
       <c r="F67" s="4"/>
       <c r="G67" s="9"/>
     </row>
-    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A68" s="8" t="s">
         <v>121</v>
       </c>
@@ -13164,7 +13227,7 @@
       </c>
       <c r="G68" s="10"/>
     </row>
-    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A69" s="4" t="s">
         <v>123</v>
       </c>
@@ -13181,7 +13244,7 @@
       </c>
       <c r="G69" s="9"/>
     </row>
-    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A70" s="8" t="s">
         <v>125</v>
       </c>
@@ -13198,7 +13261,7 @@
       </c>
       <c r="G70" s="10"/>
     </row>
-    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="4" t="s">
         <v>127</v>
       </c>
@@ -13215,7 +13278,7 @@
       </c>
       <c r="G71" s="9"/>
     </row>
-    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A72" s="8" t="s">
         <v>129</v>
       </c>
@@ -13232,7 +13295,7 @@
       </c>
       <c r="G72" s="10"/>
     </row>
-    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A73" s="4" t="s">
         <v>131</v>
       </c>
@@ -13245,7 +13308,7 @@
       <c r="F73" s="4"/>
       <c r="G73" s="9"/>
     </row>
-    <row r="74" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A74" s="8" t="s">
         <v>133</v>
       </c>
@@ -13266,7 +13329,7 @@
       </c>
       <c r="G74" s="10"/>
     </row>
-    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A75" s="4" t="s">
         <v>135</v>
       </c>
@@ -13279,7 +13342,7 @@
       <c r="F75" s="4"/>
       <c r="G75" s="9"/>
     </row>
-    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A76" s="8" t="s">
         <v>137</v>
       </c>
@@ -13296,7 +13359,7 @@
       </c>
       <c r="G76" s="10"/>
     </row>
-    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A77" s="4" t="s">
         <v>139</v>
       </c>
@@ -13311,7 +13374,7 @@
       </c>
       <c r="G77" s="9"/>
     </row>
-    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A78" s="8" t="s">
         <v>141</v>
       </c>
@@ -13324,7 +13387,7 @@
       <c r="F78" s="8"/>
       <c r="G78" s="10"/>
     </row>
-    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A79" s="4" t="s">
         <v>143</v>
       </c>
@@ -13343,7 +13406,7 @@
       </c>
       <c r="G79" s="9"/>
     </row>
-    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A80" s="8" t="s">
         <v>145</v>
       </c>
@@ -13360,7 +13423,7 @@
       </c>
       <c r="G80" s="10"/>
     </row>
-    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A81" s="4" t="s">
         <v>147</v>
       </c>
@@ -13373,7 +13436,7 @@
       <c r="F81" s="4"/>
       <c r="G81" s="9"/>
     </row>
-    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A82" s="8" t="s">
         <v>149</v>
       </c>
@@ -13386,7 +13449,7 @@
       <c r="F82" s="8"/>
       <c r="G82" s="10"/>
     </row>
-    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A83" s="4" t="s">
         <v>151</v>
       </c>
@@ -13399,7 +13462,7 @@
       <c r="F83" s="4"/>
       <c r="G83" s="9"/>
     </row>
-    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
       <c r="A84" s="8" t="s">
         <v>153</v>
       </c>
@@ -13423,15 +13486,11 @@
       <c r="B85" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C85" s="4" t="s">
-        <v>372</v>
-      </c>
+      <c r="C85" s="4"/>
       <c r="D85" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="E85" s="4" t="s">
-        <v>392</v>
-      </c>
+      <c r="E85" s="4"/>
       <c r="F85" s="4"/>
       <c r="G85" s="9"/>
     </row>
@@ -13484,14 +13543,12 @@
       <c r="D88" s="8" t="s">
         <v>407</v>
       </c>
-      <c r="E88" s="8" t="s">
-        <v>392</v>
-      </c>
+      <c r="E88" s="8"/>
       <c r="F88" s="8"/>
       <c r="G88" s="10"/>
     </row>
     <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A89" s="12" t="s">
+      <c r="A89" s="15" t="s">
         <v>163</v>
       </c>
       <c r="B89" s="4" t="s">
@@ -13556,15 +13613,11 @@
       <c r="B92" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C92" s="8" t="s">
-        <v>372</v>
-      </c>
+      <c r="C92" s="8"/>
       <c r="D92" s="8" t="s">
         <v>399</v>
       </c>
-      <c r="E92" s="8" t="s">
-        <v>392</v>
-      </c>
+      <c r="E92" s="8"/>
       <c r="F92" s="8"/>
       <c r="G92" s="10"/>
     </row>
@@ -13579,9 +13632,7 @@
       <c r="D93" s="4" t="s">
         <v>393</v>
       </c>
-      <c r="E93" s="4" t="s">
-        <v>392</v>
-      </c>
+      <c r="E93" s="4"/>
       <c r="F93" s="4"/>
       <c r="G93" s="9"/>
     </row>
@@ -13598,7 +13649,7 @@
       <c r="F94" s="8"/>
       <c r="G94" s="10"/>
     </row>
-    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="4" t="s">
         <v>175</v>
       </c>
@@ -13611,7 +13662,7 @@
       <c r="F95" s="4"/>
       <c r="G95" s="9"/>
     </row>
-    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="8" t="s">
         <v>177</v>
       </c>
@@ -13624,7 +13675,7 @@
       <c r="F96" s="8"/>
       <c r="G96" s="10"/>
     </row>
-    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="4" t="s">
         <v>179</v>
       </c>
@@ -13645,7 +13696,7 @@
       </c>
       <c r="G97" s="9"/>
     </row>
-    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="8" t="s">
         <v>181</v>
       </c>
@@ -13660,7 +13711,7 @@
       <c r="F98" s="8"/>
       <c r="G98" s="10"/>
     </row>
-    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="4" t="s">
         <v>183</v>
       </c>
@@ -13673,7 +13724,7 @@
       <c r="F99" s="4"/>
       <c r="G99" s="9"/>
     </row>
-    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="8" t="s">
         <v>185</v>
       </c>
@@ -13696,7 +13747,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="4" t="s">
         <v>187</v>
       </c>
@@ -13717,7 +13768,7 @@
       </c>
       <c r="G101" s="9"/>
     </row>
-    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="8" t="s">
         <v>189</v>
       </c>
@@ -13732,7 +13783,7 @@
       <c r="F102" s="8"/>
       <c r="G102" s="10"/>
     </row>
-    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="4" t="s">
         <v>191</v>
       </c>
@@ -13749,7 +13800,7 @@
       </c>
       <c r="G103" s="9"/>
     </row>
-    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="8" t="s">
         <v>193</v>
       </c>
@@ -13764,7 +13815,7 @@
       <c r="F104" s="8"/>
       <c r="G104" s="10"/>
     </row>
-    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="4" t="s">
         <v>195</v>
       </c>
@@ -13777,7 +13828,7 @@
       <c r="F105" s="4"/>
       <c r="G105" s="9"/>
     </row>
-    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="8" t="s">
         <v>197</v>
       </c>
@@ -13790,7 +13841,7 @@
       <c r="F106" s="8"/>
       <c r="G106" s="10"/>
     </row>
-    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A107" s="4" t="s">
         <v>199</v>
       </c>
@@ -13811,7 +13862,7 @@
       </c>
       <c r="G107" s="9"/>
     </row>
-    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="8" t="s">
         <v>201</v>
       </c>
@@ -13830,7 +13881,7 @@
       </c>
       <c r="G108" s="10"/>
     </row>
-    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A109" s="4" t="s">
         <v>203</v>
       </c>
@@ -13853,7 +13904,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="8" t="s">
         <v>205</v>
       </c>
@@ -13872,7 +13923,7 @@
       </c>
       <c r="G110" s="10"/>
     </row>
-    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A111" s="4" t="s">
         <v>207</v>
       </c>
@@ -13887,7 +13938,7 @@
       <c r="F111" s="4"/>
       <c r="G111" s="9"/>
     </row>
-    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A112" s="8" t="s">
         <v>209</v>
       </c>
@@ -13900,7 +13951,7 @@
       <c r="F112" s="8"/>
       <c r="G112" s="10"/>
     </row>
-    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A113" s="4" t="s">
         <v>211</v>
       </c>
@@ -13932,9 +13983,7 @@
       <c r="D114" s="8" t="s">
         <v>406</v>
       </c>
-      <c r="E114" s="8" t="s">
-        <v>392</v>
-      </c>
+      <c r="E114" s="8"/>
       <c r="F114" s="8"/>
       <c r="G114" s="10"/>
     </row>
@@ -13962,9 +14011,7 @@
       <c r="D116" s="8" t="s">
         <v>397</v>
       </c>
-      <c r="E116" s="8" t="s">
-        <v>392</v>
-      </c>
+      <c r="E116" s="8"/>
       <c r="F116" s="8"/>
       <c r="G116" s="10"/>
     </row>
@@ -13975,15 +14022,11 @@
       <c r="B117" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="C117" s="4" t="s">
-        <v>372</v>
-      </c>
+      <c r="C117" s="4"/>
       <c r="D117" s="4" t="s">
         <v>395</v>
       </c>
-      <c r="E117" s="4" t="s">
-        <v>392</v>
-      </c>
+      <c r="E117" s="4"/>
       <c r="F117" s="4"/>
       <c r="G117" s="9"/>
     </row>
@@ -13998,9 +14041,7 @@
       <c r="D118" s="8" t="s">
         <v>404</v>
       </c>
-      <c r="E118" s="8" t="s">
-        <v>392</v>
-      </c>
+      <c r="E118" s="8"/>
       <c r="F118" s="8"/>
       <c r="G118" s="10"/>
     </row>
@@ -14011,15 +14052,11 @@
       <c r="B119" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="C119" s="4" t="s">
-        <v>372</v>
-      </c>
+      <c r="C119" s="4"/>
       <c r="D119" s="4" t="s">
         <v>401</v>
       </c>
-      <c r="E119" s="4" t="s">
-        <v>392</v>
-      </c>
+      <c r="E119" s="4"/>
       <c r="F119" s="4"/>
       <c r="G119" s="9"/>
     </row>
@@ -14030,15 +14067,11 @@
       <c r="B120" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="C120" s="8" t="s">
-        <v>372</v>
-      </c>
+      <c r="C120" s="8"/>
       <c r="D120" s="8" t="s">
         <v>396</v>
       </c>
-      <c r="E120" s="8" t="s">
-        <v>392</v>
-      </c>
+      <c r="E120" s="8"/>
       <c r="F120" s="8"/>
       <c r="G120" s="10"/>
     </row>
@@ -14053,9 +14086,7 @@
       <c r="D121" s="4" t="s">
         <v>390</v>
       </c>
-      <c r="E121" s="4" t="s">
-        <v>392</v>
-      </c>
+      <c r="E121" s="4"/>
       <c r="F121" s="4"/>
       <c r="G121" s="9"/>
     </row>
@@ -14097,7 +14128,7 @@
       <c r="F123" s="4"/>
       <c r="G123" s="9"/>
     </row>
-    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="8" t="s">
         <v>233</v>
       </c>
@@ -14110,7 +14141,7 @@
       <c r="F124" s="8"/>
       <c r="G124" s="10"/>
     </row>
-    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="4" t="s">
         <v>235</v>
       </c>
@@ -14127,7 +14158,7 @@
       </c>
       <c r="G125" s="9"/>
     </row>
-    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="8" t="s">
         <v>237</v>
       </c>
@@ -14140,7 +14171,7 @@
       <c r="F126" s="8"/>
       <c r="G126" s="10"/>
     </row>
-    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="4" t="s">
         <v>239</v>
       </c>
@@ -14161,7 +14192,7 @@
       </c>
       <c r="G127" s="9"/>
     </row>
-    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="8" t="s">
         <v>241</v>
       </c>
@@ -14178,7 +14209,7 @@
       </c>
       <c r="G128" s="10"/>
     </row>
-    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="4" t="s">
         <v>243</v>
       </c>
@@ -14193,7 +14224,7 @@
       <c r="F129" s="4"/>
       <c r="G129" s="9"/>
     </row>
-    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="8" t="s">
         <v>245</v>
       </c>
@@ -14210,7 +14241,7 @@
       </c>
       <c r="G130" s="10"/>
     </row>
-    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="4" t="s">
         <v>247</v>
       </c>
@@ -14223,7 +14254,7 @@
       <c r="F131" s="4"/>
       <c r="G131" s="9"/>
     </row>
-    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="8" t="s">
         <v>249</v>
       </c>
@@ -14246,7 +14277,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="4" t="s">
         <v>251</v>
       </c>
@@ -14261,7 +14292,7 @@
       <c r="F133" s="4"/>
       <c r="G133" s="9"/>
     </row>
-    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="8" t="s">
         <v>253</v>
       </c>
@@ -14282,7 +14313,7 @@
       </c>
       <c r="G134" s="10"/>
     </row>
-    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="4" t="s">
         <v>255</v>
       </c>
@@ -14303,7 +14334,7 @@
       </c>
       <c r="G135" s="9"/>
     </row>
-    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A136" s="8" t="s">
         <v>257</v>
       </c>
@@ -14318,7 +14349,7 @@
       <c r="F136" s="8"/>
       <c r="G136" s="10"/>
     </row>
-    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A137" s="4" t="s">
         <v>259</v>
       </c>
@@ -14339,7 +14370,7 @@
       </c>
       <c r="G137" s="9"/>
     </row>
-    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A138" s="8" t="s">
         <v>261</v>
       </c>
@@ -14360,7 +14391,7 @@
       </c>
       <c r="G138" s="10"/>
     </row>
-    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A139" s="4" t="s">
         <v>263</v>
       </c>
@@ -14381,7 +14412,7 @@
       </c>
       <c r="G139" s="9"/>
     </row>
-    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A140" s="8" t="s">
         <v>265</v>
       </c>
@@ -14394,7 +14425,7 @@
       <c r="F140" s="8"/>
       <c r="G140" s="10"/>
     </row>
-    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A141" s="4" t="s">
         <v>267</v>
       </c>
@@ -14407,7 +14438,7 @@
       <c r="F141" s="4"/>
       <c r="G141" s="9"/>
     </row>
-    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="8" t="s">
         <v>269</v>
       </c>
@@ -14424,7 +14455,7 @@
       </c>
       <c r="G142" s="10"/>
     </row>
-    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A143" s="4" t="s">
         <v>271</v>
       </c>
@@ -14437,7 +14468,7 @@
       <c r="F143" s="4"/>
       <c r="G143" s="9"/>
     </row>
-    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A144" s="8" t="s">
         <v>273</v>
       </c>
@@ -14454,7 +14485,7 @@
       </c>
       <c r="G144" s="10"/>
     </row>
-    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A145" s="4" t="s">
         <v>275</v>
       </c>
@@ -14467,7 +14498,7 @@
       <c r="F145" s="4"/>
       <c r="G145" s="9"/>
     </row>
-    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A146" s="8" t="s">
         <v>277</v>
       </c>
@@ -14480,7 +14511,7 @@
       <c r="F146" s="8"/>
       <c r="G146" s="10"/>
     </row>
-    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A147" s="4" t="s">
         <v>279</v>
       </c>
@@ -14491,7 +14522,7 @@
       <c r="F147" s="4"/>
       <c r="G147" s="9"/>
     </row>
-    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A148" s="8" t="s">
         <v>281</v>
       </c>
@@ -14504,7 +14535,7 @@
       <c r="F148" s="8"/>
       <c r="G148" s="10"/>
     </row>
-    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A149" s="4" t="s">
         <v>283</v>
       </c>
@@ -14517,7 +14548,7 @@
       <c r="F149" s="4"/>
       <c r="G149" s="9"/>
     </row>
-    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A150" s="8" t="s">
         <v>285</v>
       </c>
@@ -14530,7 +14561,7 @@
       <c r="F150" s="8"/>
       <c r="G150" s="10"/>
     </row>
-    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A151" s="4" t="s">
         <v>287</v>
       </c>
@@ -14543,7 +14574,7 @@
       <c r="F151" s="4"/>
       <c r="G151" s="9"/>
     </row>
-    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A152" s="8" t="s">
         <v>289</v>
       </c>
@@ -14566,6 +14597,2744 @@
       <c r="C153" s="4"/>
       <c r="D153" s="4"/>
       <c r="E153" s="4"/>
+      <c r="F153" s="4"/>
+      <c r="G153" s="9"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C154" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D154" s="8"/>
+      <c r="E154" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F154" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="10"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4"/>
+      <c r="G155" s="9"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C156" s="8"/>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8"/>
+      <c r="F156" s="8"/>
+      <c r="G156" s="10"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C157" s="4"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4"/>
+      <c r="G157" s="9"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B158" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C158" s="8"/>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8"/>
+      <c r="F158" s="8"/>
+      <c r="G158" s="10"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="9"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B160" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C160" s="8"/>
+      <c r="D160" s="8"/>
+      <c r="E160" s="8"/>
+      <c r="F160" s="8"/>
+      <c r="G160" s="10"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+      <c r="G161" s="9"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B162" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C162" s="8"/>
+      <c r="D162" s="8"/>
+      <c r="E162" s="8"/>
+      <c r="F162" s="8"/>
+      <c r="G162" s="10"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+      <c r="G163" s="9"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B164" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C164" s="8"/>
+      <c r="D164" s="8"/>
+      <c r="E164" s="8"/>
+      <c r="F164" s="8"/>
+      <c r="G164" s="10"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C165" s="4"/>
+      <c r="D165" s="4"/>
+      <c r="E165" s="4"/>
+      <c r="F165" s="4"/>
+      <c r="G165" s="9"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B166" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C166" s="8"/>
+      <c r="D166" s="8"/>
+      <c r="E166" s="8"/>
+      <c r="F166" s="8"/>
+      <c r="G166" s="10"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D167" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E167" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G167" s="9"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B168" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C168" s="8"/>
+      <c r="D168" s="8"/>
+      <c r="E168" s="8"/>
+      <c r="F168" s="8"/>
+      <c r="G168" s="10"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C169" s="4"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="9"/>
+    </row>
+    <row r="170" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A170" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B170" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C170" s="8"/>
+      <c r="D170" s="8"/>
+      <c r="E170" s="8"/>
+      <c r="F170" s="8"/>
+      <c r="G170" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G170" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="CAÇAMBA IVECO 28260 PL PIG 5304 POTY"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS  SR004989 PLACA SLT 6C49"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS R002697 PLACA SLT 6D33"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR002618 PLACA SLT 6D30"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR002652 PLACA SLT 6D34"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR002658 PLACA SLT 6D25"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR004619 PLACA SLT 6C45"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR005043 PLACA SLT 6C48"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR005574 PLACA SLT 6C43"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR005579 PLACA SLT 6C50"/>
+        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR005705 PLACA SLT 6C44"/>
+        <filter val="CAÇAMBA NOVA VW 26330 Chassi: 9536C8TD8RR058330 | DANFE 618388 SLR 6C65"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058361 PLACA SLR-0E27"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058408 PLACA SLR-4G15"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058635 PLACA SLR-4G25"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058697 PLACA SLR-4E18"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058778 PLACA SLR-4G29"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058862 PLACA SLR-0i11"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR059087 PLACA SLR-0E23"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR059154 PLACA SLR-0E26"/>
+        <filter val="CAÇAMBA NOVA VW 26330 CHSSISRR058957 PLACA SLR-0E19"/>
+        <filter val="CAÇAMBA SCANEA 310 PL PIN 0144 POTY"/>
+        <filter val="CAÇAMBA VOLKS 24260 PL QRR 5B87 POTY"/>
+        <filter val="CAÇAMBA VOLKS 24260 PL QRR 8A07 POTY"/>
+        <filter val="CAÇAMBA VOLVO 270 PL PIZ 3804 POTY"/>
+        <filter val="CAÇAMBA VOLVO 270 PL PIZ 3i14 POTY"/>
+        <filter val="CAÇAMBA VOLVO 330 PL QRR 4G34 POTY"/>
+        <filter val="CAÇAMBÃO COLOM  PLACA PIA 7B52"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93CBAED5-FEB5-44AD-8E39-A42A39B23940}">
+  <dimension ref="A1:G170"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
+        <v>416</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="10"/>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F54" s="8"/>
+      <c r="G54" s="10"/>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F56" s="8"/>
+      <c r="G56" s="10"/>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F57" s="4"/>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F58" s="8"/>
+      <c r="G58" s="10"/>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F59" s="4"/>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="10"/>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8"/>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10"/>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="9"/>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8"/>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8"/>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="8"/>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10"/>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8"/>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8"/>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F85" s="4"/>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F86" s="8"/>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F87" s="4"/>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F88" s="8"/>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F90" s="8"/>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F91" s="4"/>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F92" s="8"/>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F93" s="4"/>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F94" s="8"/>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+      <c r="F95" s="4"/>
+      <c r="G95" s="9"/>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="8"/>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8"/>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8"/>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+      <c r="F105" s="4"/>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8"/>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8"/>
+      <c r="F106" s="8"/>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8"/>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="C112" s="8"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="8"/>
+      <c r="G112" s="10"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E113" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="9"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C114" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D114" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F114" s="8"/>
+      <c r="G114" s="10"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D115" s="4"/>
+      <c r="E115" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F115" s="4"/>
+      <c r="G115" s="9"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C116" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D116" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F116" s="8"/>
+      <c r="G116" s="10"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D117" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E117" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F117" s="4"/>
+      <c r="G117" s="9"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B118" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C118" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D118" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F118" s="8"/>
+      <c r="G118" s="10"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D119" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E119" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F119" s="4"/>
+      <c r="G119" s="9"/>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C120" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D120" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F120" s="8"/>
+      <c r="G120" s="10"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D121" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E121" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F121" s="4"/>
+      <c r="G121" s="9"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B122" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C122" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E122" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F122" s="8"/>
+      <c r="G122" s="10"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E123" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F123" s="4"/>
+      <c r="G123" s="9"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B124" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C124" s="8"/>
+      <c r="D124" s="8"/>
+      <c r="E124" s="8"/>
+      <c r="F124" s="8"/>
+      <c r="G124" s="10"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D125" s="4"/>
+      <c r="E125" s="4"/>
+      <c r="F125" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G125" s="9"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C126" s="8"/>
+      <c r="D126" s="8"/>
+      <c r="E126" s="8"/>
+      <c r="F126" s="8"/>
+      <c r="G126" s="10"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E127" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G127" s="9"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C128" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="8"/>
+      <c r="E128" s="8"/>
+      <c r="F128" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G128" s="10"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="4"/>
+      <c r="E129" s="4"/>
+      <c r="F129" s="4"/>
+      <c r="G129" s="9"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="8"/>
+      <c r="E130" s="8"/>
+      <c r="F130" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G130" s="10"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C131" s="4"/>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+      <c r="G131" s="9"/>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D132" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F132" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D133" s="4"/>
+      <c r="E133" s="4"/>
+      <c r="F133" s="4"/>
+      <c r="G133" s="9"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C134" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D134" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F134" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="10"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E135" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G135" s="9"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C136" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D136" s="8"/>
+      <c r="E136" s="8"/>
+      <c r="F136" s="8"/>
+      <c r="G136" s="10"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E137" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="9"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C138" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D138" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F138" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="10"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D139" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E139" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G139" s="9"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C140" s="8"/>
+      <c r="D140" s="8"/>
+      <c r="E140" s="8"/>
+      <c r="F140" s="8"/>
+      <c r="G140" s="10"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C141" s="4"/>
+      <c r="D141" s="4"/>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="9"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C142" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="8"/>
+      <c r="E142" s="8"/>
+      <c r="F142" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G142" s="10"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4"/>
+      <c r="G143" s="9"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="8"/>
+      <c r="E144" s="8"/>
+      <c r="F144" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G144" s="10"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C145" s="4"/>
+      <c r="D145" s="4"/>
+      <c r="E145" s="4"/>
+      <c r="F145" s="4"/>
+      <c r="G145" s="9"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B146" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C146" s="8"/>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8"/>
+      <c r="G146" s="10"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="E147" s="4"/>
+      <c r="F147" s="4"/>
+      <c r="G147" s="9"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B148" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C148" s="8"/>
+      <c r="D148" s="8"/>
+      <c r="E148" s="8"/>
+      <c r="F148" s="8"/>
+      <c r="G148" s="10"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C149" s="4"/>
+      <c r="D149" s="4"/>
+      <c r="E149" s="4"/>
+      <c r="F149" s="4"/>
+      <c r="G149" s="9"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C150" s="8"/>
+      <c r="D150" s="8"/>
+      <c r="E150" s="8"/>
+      <c r="F150" s="8"/>
+      <c r="G150" s="10"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="9"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B152" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C152" s="8"/>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
+      <c r="F152" s="8"/>
+      <c r="G152" s="10"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C153" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D153" s="4"/>
+      <c r="E153" s="4" t="s">
+        <v>392</v>
+      </c>
       <c r="F153" s="4"/>
       <c r="G153" s="9"/>
     </row>

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA MARÇO: CHECKLIST 19/03 11:22h
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C71F5B9-01A1-453D-8261-D0013660BF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E09335-069C-480F-9703-F0893F7097BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="17" sheetId="5" r:id="rId4"/>
     <sheet name="18" sheetId="6" r:id="rId5"/>
     <sheet name="19" sheetId="7" r:id="rId6"/>
+    <sheet name="20" sheetId="8" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
@@ -27,6 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'17'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'18'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'19'!$A$6:$G$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'20'!$A$6:$G$170</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3056" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3755" uniqueCount="425">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1300,6 +1302,30 @@
   </si>
   <si>
     <t>DATA DA CONFERENCIA: 19/03/2026</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERENCIA: 20/03/2026</t>
+  </si>
+  <si>
+    <t>FORTALEZA</t>
+  </si>
+  <si>
+    <t>TRANSITO</t>
+  </si>
+  <si>
+    <t>VENDIDA</t>
+  </si>
+  <si>
+    <t>OFICINA - MONACO</t>
+  </si>
+  <si>
+    <t>PRF</t>
+  </si>
+  <si>
+    <t>OFICINA - TERCEIRIZADA</t>
+  </si>
+  <si>
+    <t>DEVOLVIDA</t>
   </si>
 </sst>
 </file>
@@ -1313,7 +1339,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1350,6 +1376,12 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="7"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="7"/>
       <name val="Verdana"/>
       <family val="2"/>
@@ -1487,9 +1519,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
@@ -1803,6 +1833,59 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D46519E0-8A5D-41CE-9640-961A613AA8FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D57DAFAC-94F7-4479-A43C-9371A84ED3F1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -12219,7 +12302,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{255AD8CD-DB98-4F1E-AEC5-D12CAEE762DC}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G170"/>
   <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
@@ -12297,7 +12379,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A7" s="4" t="s">
         <v>0</v>
       </c>
@@ -12314,7 +12396,7 @@
       </c>
       <c r="G7" s="9"/>
     </row>
-    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A8" s="8" t="s">
         <v>2</v>
       </c>
@@ -12329,7 +12411,7 @@
       <c r="F8" s="8"/>
       <c r="G8" s="10"/>
     </row>
-    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A9" s="4" t="s">
         <v>4</v>
       </c>
@@ -12346,7 +12428,7 @@
       </c>
       <c r="G9" s="9"/>
     </row>
-    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A10" s="8" t="s">
         <v>6</v>
       </c>
@@ -12359,7 +12441,7 @@
       <c r="F10" s="8"/>
       <c r="G10" s="10"/>
     </row>
-    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
@@ -12376,7 +12458,7 @@
       </c>
       <c r="G11" s="9"/>
     </row>
-    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A12" s="8" t="s">
         <v>10</v>
       </c>
@@ -12389,7 +12471,7 @@
       <c r="F12" s="8"/>
       <c r="G12" s="10"/>
     </row>
-    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
@@ -12406,7 +12488,7 @@
       </c>
       <c r="G13" s="9"/>
     </row>
-    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A14" s="8" t="s">
         <v>14</v>
       </c>
@@ -12423,7 +12505,7 @@
       </c>
       <c r="G14" s="10"/>
     </row>
-    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
@@ -12440,7 +12522,7 @@
       </c>
       <c r="G15" s="9"/>
     </row>
-    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A16" s="8" t="s">
         <v>18</v>
       </c>
@@ -12455,7 +12537,7 @@
       <c r="F16" s="8"/>
       <c r="G16" s="10"/>
     </row>
-    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
@@ -12468,7 +12550,7 @@
       <c r="F17" s="4"/>
       <c r="G17" s="9"/>
     </row>
-    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
@@ -12481,7 +12563,7 @@
       <c r="F18" s="8"/>
       <c r="G18" s="10"/>
     </row>
-    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A19" s="4" t="s">
         <v>24</v>
       </c>
@@ -12494,7 +12576,7 @@
       <c r="F19" s="4"/>
       <c r="G19" s="9"/>
     </row>
-    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A20" s="8" t="s">
         <v>26</v>
       </c>
@@ -12507,7 +12589,7 @@
       <c r="F20" s="8"/>
       <c r="G20" s="10"/>
     </row>
-    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A21" s="4" t="s">
         <v>28</v>
       </c>
@@ -12522,7 +12604,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="9"/>
     </row>
-    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A22" s="8" t="s">
         <v>30</v>
       </c>
@@ -12539,7 +12621,7 @@
       </c>
       <c r="G22" s="10"/>
     </row>
-    <row r="23" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A23" s="4" t="s">
         <v>32</v>
       </c>
@@ -12560,7 +12642,7 @@
       </c>
       <c r="G23" s="9"/>
     </row>
-    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A24" s="8" t="s">
         <v>34</v>
       </c>
@@ -12573,7 +12655,7 @@
       <c r="F24" s="8"/>
       <c r="G24" s="10"/>
     </row>
-    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A25" s="4" t="s">
         <v>36</v>
       </c>
@@ -12590,7 +12672,7 @@
       </c>
       <c r="G25" s="9"/>
     </row>
-    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A26" s="8" t="s">
         <v>38</v>
       </c>
@@ -12607,7 +12689,7 @@
       </c>
       <c r="G26" s="10"/>
     </row>
-    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A27" s="4" t="s">
         <v>40</v>
       </c>
@@ -12624,7 +12706,7 @@
       </c>
       <c r="G27" s="9"/>
     </row>
-    <row r="28" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A28" s="8" t="s">
         <v>42</v>
       </c>
@@ -12645,7 +12727,7 @@
       </c>
       <c r="G28" s="10"/>
     </row>
-    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A29" s="4" t="s">
         <v>44</v>
       </c>
@@ -12658,7 +12740,7 @@
       <c r="F29" s="4"/>
       <c r="G29" s="9"/>
     </row>
-    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A30" s="8" t="s">
         <v>46</v>
       </c>
@@ -12671,7 +12753,7 @@
       <c r="F30" s="8"/>
       <c r="G30" s="10"/>
     </row>
-    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="4" t="s">
         <v>48</v>
       </c>
@@ -12684,7 +12766,7 @@
       <c r="F31" s="4"/>
       <c r="G31" s="9"/>
     </row>
-    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A32" s="8" t="s">
         <v>50</v>
       </c>
@@ -12697,7 +12779,7 @@
       <c r="F32" s="8"/>
       <c r="G32" s="10"/>
     </row>
-    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A33" s="4" t="s">
         <v>52</v>
       </c>
@@ -12710,7 +12792,7 @@
       <c r="F33" s="4"/>
       <c r="G33" s="9"/>
     </row>
-    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A34" s="8" t="s">
         <v>54</v>
       </c>
@@ -12723,7 +12805,7 @@
       <c r="F34" s="8"/>
       <c r="G34" s="10"/>
     </row>
-    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="4" t="s">
         <v>56</v>
       </c>
@@ -12746,7 +12828,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A36" s="8" t="s">
         <v>58</v>
       </c>
@@ -12759,7 +12841,7 @@
       <c r="F36" s="8"/>
       <c r="G36" s="10"/>
     </row>
-    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A37" s="4" t="s">
         <v>60</v>
       </c>
@@ -12772,7 +12854,7 @@
       <c r="F37" s="4"/>
       <c r="G37" s="9"/>
     </row>
-    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A38" s="8" t="s">
         <v>62</v>
       </c>
@@ -12785,7 +12867,7 @@
       <c r="F38" s="8"/>
       <c r="G38" s="10"/>
     </row>
-    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A39" s="4" t="s">
         <v>64</v>
       </c>
@@ -12798,7 +12880,7 @@
       <c r="F39" s="4"/>
       <c r="G39" s="9"/>
     </row>
-    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A40" s="8" t="s">
         <v>66</v>
       </c>
@@ -12811,7 +12893,7 @@
       <c r="F40" s="8"/>
       <c r="G40" s="10"/>
     </row>
-    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A41" s="4" t="s">
         <v>68</v>
       </c>
@@ -12824,7 +12906,7 @@
       <c r="F41" s="4"/>
       <c r="G41" s="9"/>
     </row>
-    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A42" s="8" t="s">
         <v>70</v>
       </c>
@@ -12837,7 +12919,7 @@
       <c r="F42" s="8"/>
       <c r="G42" s="10"/>
     </row>
-    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A43" s="4" t="s">
         <v>72</v>
       </c>
@@ -12850,7 +12932,7 @@
       <c r="F43" s="4"/>
       <c r="G43" s="9"/>
     </row>
-    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A44" s="8" t="s">
         <v>74</v>
       </c>
@@ -12863,7 +12945,7 @@
       <c r="F44" s="8"/>
       <c r="G44" s="10"/>
     </row>
-    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A45" s="4" t="s">
         <v>76</v>
       </c>
@@ -12876,7 +12958,7 @@
       <c r="F45" s="4"/>
       <c r="G45" s="9"/>
     </row>
-    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A46" s="8" t="s">
         <v>78</v>
       </c>
@@ -12895,7 +12977,7 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A47" s="4" t="s">
         <v>80</v>
       </c>
@@ -12908,7 +12990,7 @@
       <c r="F47" s="4"/>
       <c r="G47" s="9"/>
     </row>
-    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A48" s="8" t="s">
         <v>82</v>
       </c>
@@ -12921,7 +13003,7 @@
       <c r="F48" s="8"/>
       <c r="G48" s="10"/>
     </row>
-    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A49" s="4" t="s">
         <v>84</v>
       </c>
@@ -12934,7 +13016,7 @@
       <c r="F49" s="4"/>
       <c r="G49" s="9"/>
     </row>
-    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A50" s="8" t="s">
         <v>86</v>
       </c>
@@ -12947,7 +13029,7 @@
       <c r="F50" s="8"/>
       <c r="G50" s="10"/>
     </row>
-    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" hidden="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A51" s="4" t="s">
         <v>88</v>
       </c>
@@ -12964,7 +13046,7 @@
       </c>
       <c r="G51" s="9"/>
     </row>
-    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A52" s="8" t="s">
         <v>90</v>
       </c>
@@ -12977,7 +13059,7 @@
       <c r="F52" s="8"/>
       <c r="G52" s="10"/>
     </row>
-    <row r="53" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A53" s="4" t="s">
         <v>91</v>
       </c>
@@ -13011,7 +13093,7 @@
       <c r="F54" s="8"/>
       <c r="G54" s="10"/>
     </row>
-    <row r="55" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A55" s="4" t="s">
         <v>95</v>
       </c>
@@ -13086,7 +13168,7 @@
       <c r="F59" s="4"/>
       <c r="G59" s="9"/>
     </row>
-    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A60" s="8" t="s">
         <v>105</v>
       </c>
@@ -13099,7 +13181,7 @@
       <c r="F60" s="8"/>
       <c r="G60" s="10"/>
     </row>
-    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A61" s="4" t="s">
         <v>107</v>
       </c>
@@ -13112,7 +13194,7 @@
       <c r="F61" s="4"/>
       <c r="G61" s="9"/>
     </row>
-    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A62" s="8" t="s">
         <v>109</v>
       </c>
@@ -13125,7 +13207,7 @@
       <c r="F62" s="8"/>
       <c r="G62" s="10"/>
     </row>
-    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A63" s="4" t="s">
         <v>111</v>
       </c>
@@ -13142,7 +13224,7 @@
       </c>
       <c r="G63" s="9"/>
     </row>
-    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A64" s="8" t="s">
         <v>113</v>
       </c>
@@ -13159,7 +13241,7 @@
       </c>
       <c r="G64" s="10"/>
     </row>
-    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A65" s="4" t="s">
         <v>115</v>
       </c>
@@ -13176,7 +13258,7 @@
       </c>
       <c r="G65" s="9"/>
     </row>
-    <row r="66" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A66" s="8" t="s">
         <v>117</v>
       </c>
@@ -13197,7 +13279,7 @@
       </c>
       <c r="G66" s="10"/>
     </row>
-    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A67" s="4" t="s">
         <v>119</v>
       </c>
@@ -13210,7 +13292,7 @@
       <c r="F67" s="4"/>
       <c r="G67" s="9"/>
     </row>
-    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A68" s="8" t="s">
         <v>121</v>
       </c>
@@ -13227,7 +13309,7 @@
       </c>
       <c r="G68" s="10"/>
     </row>
-    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A69" s="4" t="s">
         <v>123</v>
       </c>
@@ -13244,7 +13326,7 @@
       </c>
       <c r="G69" s="9"/>
     </row>
-    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A70" s="8" t="s">
         <v>125</v>
       </c>
@@ -13261,7 +13343,7 @@
       </c>
       <c r="G70" s="10"/>
     </row>
-    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="4" t="s">
         <v>127</v>
       </c>
@@ -13278,7 +13360,7 @@
       </c>
       <c r="G71" s="9"/>
     </row>
-    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A72" s="8" t="s">
         <v>129</v>
       </c>
@@ -13295,7 +13377,7 @@
       </c>
       <c r="G72" s="10"/>
     </row>
-    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A73" s="4" t="s">
         <v>131</v>
       </c>
@@ -13308,7 +13390,7 @@
       <c r="F73" s="4"/>
       <c r="G73" s="9"/>
     </row>
-    <row r="74" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A74" s="8" t="s">
         <v>133</v>
       </c>
@@ -13329,7 +13411,7 @@
       </c>
       <c r="G74" s="10"/>
     </row>
-    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A75" s="4" t="s">
         <v>135</v>
       </c>
@@ -13342,7 +13424,7 @@
       <c r="F75" s="4"/>
       <c r="G75" s="9"/>
     </row>
-    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A76" s="8" t="s">
         <v>137</v>
       </c>
@@ -13359,7 +13441,7 @@
       </c>
       <c r="G76" s="10"/>
     </row>
-    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A77" s="4" t="s">
         <v>139</v>
       </c>
@@ -13374,7 +13456,7 @@
       </c>
       <c r="G77" s="9"/>
     </row>
-    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A78" s="8" t="s">
         <v>141</v>
       </c>
@@ -13387,7 +13469,7 @@
       <c r="F78" s="8"/>
       <c r="G78" s="10"/>
     </row>
-    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A79" s="4" t="s">
         <v>143</v>
       </c>
@@ -13406,7 +13488,7 @@
       </c>
       <c r="G79" s="9"/>
     </row>
-    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A80" s="8" t="s">
         <v>145</v>
       </c>
@@ -13423,7 +13505,7 @@
       </c>
       <c r="G80" s="10"/>
     </row>
-    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A81" s="4" t="s">
         <v>147</v>
       </c>
@@ -13436,7 +13518,7 @@
       <c r="F81" s="4"/>
       <c r="G81" s="9"/>
     </row>
-    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A82" s="8" t="s">
         <v>149</v>
       </c>
@@ -13449,7 +13531,7 @@
       <c r="F82" s="8"/>
       <c r="G82" s="10"/>
     </row>
-    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A83" s="4" t="s">
         <v>151</v>
       </c>
@@ -13462,7 +13544,7 @@
       <c r="F83" s="4"/>
       <c r="G83" s="9"/>
     </row>
-    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" hidden="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A84" s="8" t="s">
         <v>153</v>
       </c>
@@ -13548,7 +13630,7 @@
       <c r="G88" s="10"/>
     </row>
     <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A89" s="15" t="s">
+      <c r="A89" s="4" t="s">
         <v>163</v>
       </c>
       <c r="B89" s="4" t="s">
@@ -13649,7 +13731,7 @@
       <c r="F94" s="8"/>
       <c r="G94" s="10"/>
     </row>
-    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="4" t="s">
         <v>175</v>
       </c>
@@ -13662,7 +13744,7 @@
       <c r="F95" s="4"/>
       <c r="G95" s="9"/>
     </row>
-    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="8" t="s">
         <v>177</v>
       </c>
@@ -13675,7 +13757,7 @@
       <c r="F96" s="8"/>
       <c r="G96" s="10"/>
     </row>
-    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="4" t="s">
         <v>179</v>
       </c>
@@ -13696,7 +13778,7 @@
       </c>
       <c r="G97" s="9"/>
     </row>
-    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="8" t="s">
         <v>181</v>
       </c>
@@ -13711,7 +13793,7 @@
       <c r="F98" s="8"/>
       <c r="G98" s="10"/>
     </row>
-    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="4" t="s">
         <v>183</v>
       </c>
@@ -13724,7 +13806,7 @@
       <c r="F99" s="4"/>
       <c r="G99" s="9"/>
     </row>
-    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="8" t="s">
         <v>185</v>
       </c>
@@ -13747,7 +13829,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="4" t="s">
         <v>187</v>
       </c>
@@ -13768,7 +13850,7 @@
       </c>
       <c r="G101" s="9"/>
     </row>
-    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="8" t="s">
         <v>189</v>
       </c>
@@ -13783,7 +13865,7 @@
       <c r="F102" s="8"/>
       <c r="G102" s="10"/>
     </row>
-    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="4" t="s">
         <v>191</v>
       </c>
@@ -13800,7 +13882,7 @@
       </c>
       <c r="G103" s="9"/>
     </row>
-    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="8" t="s">
         <v>193</v>
       </c>
@@ -13815,7 +13897,7 @@
       <c r="F104" s="8"/>
       <c r="G104" s="10"/>
     </row>
-    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="4" t="s">
         <v>195</v>
       </c>
@@ -13828,7 +13910,7 @@
       <c r="F105" s="4"/>
       <c r="G105" s="9"/>
     </row>
-    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="8" t="s">
         <v>197</v>
       </c>
@@ -13841,7 +13923,7 @@
       <c r="F106" s="8"/>
       <c r="G106" s="10"/>
     </row>
-    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A107" s="4" t="s">
         <v>199</v>
       </c>
@@ -13862,7 +13944,7 @@
       </c>
       <c r="G107" s="9"/>
     </row>
-    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="8" t="s">
         <v>201</v>
       </c>
@@ -13881,7 +13963,7 @@
       </c>
       <c r="G108" s="10"/>
     </row>
-    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A109" s="4" t="s">
         <v>203</v>
       </c>
@@ -13904,7 +13986,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="8" t="s">
         <v>205</v>
       </c>
@@ -13923,7 +14005,7 @@
       </c>
       <c r="G110" s="10"/>
     </row>
-    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A111" s="4" t="s">
         <v>207</v>
       </c>
@@ -13938,7 +14020,7 @@
       <c r="F111" s="4"/>
       <c r="G111" s="9"/>
     </row>
-    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A112" s="8" t="s">
         <v>209</v>
       </c>
@@ -13951,7 +14033,7 @@
       <c r="F112" s="8"/>
       <c r="G112" s="10"/>
     </row>
-    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A113" s="4" t="s">
         <v>211</v>
       </c>
@@ -14128,7 +14210,7 @@
       <c r="F123" s="4"/>
       <c r="G123" s="9"/>
     </row>
-    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="8" t="s">
         <v>233</v>
       </c>
@@ -14141,7 +14223,7 @@
       <c r="F124" s="8"/>
       <c r="G124" s="10"/>
     </row>
-    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="4" t="s">
         <v>235</v>
       </c>
@@ -14158,7 +14240,7 @@
       </c>
       <c r="G125" s="9"/>
     </row>
-    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="8" t="s">
         <v>237</v>
       </c>
@@ -14171,7 +14253,7 @@
       <c r="F126" s="8"/>
       <c r="G126" s="10"/>
     </row>
-    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="4" t="s">
         <v>239</v>
       </c>
@@ -14192,7 +14274,7 @@
       </c>
       <c r="G127" s="9"/>
     </row>
-    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="8" t="s">
         <v>241</v>
       </c>
@@ -14209,7 +14291,7 @@
       </c>
       <c r="G128" s="10"/>
     </row>
-    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="4" t="s">
         <v>243</v>
       </c>
@@ -14224,7 +14306,7 @@
       <c r="F129" s="4"/>
       <c r="G129" s="9"/>
     </row>
-    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="8" t="s">
         <v>245</v>
       </c>
@@ -14241,7 +14323,7 @@
       </c>
       <c r="G130" s="10"/>
     </row>
-    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="4" t="s">
         <v>247</v>
       </c>
@@ -14254,7 +14336,7 @@
       <c r="F131" s="4"/>
       <c r="G131" s="9"/>
     </row>
-    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="8" t="s">
         <v>249</v>
       </c>
@@ -14277,7 +14359,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="4" t="s">
         <v>251</v>
       </c>
@@ -14292,7 +14374,7 @@
       <c r="F133" s="4"/>
       <c r="G133" s="9"/>
     </row>
-    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="8" t="s">
         <v>253</v>
       </c>
@@ -14313,7 +14395,7 @@
       </c>
       <c r="G134" s="10"/>
     </row>
-    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="4" t="s">
         <v>255</v>
       </c>
@@ -14334,7 +14416,7 @@
       </c>
       <c r="G135" s="9"/>
     </row>
-    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A136" s="8" t="s">
         <v>257</v>
       </c>
@@ -14349,7 +14431,7 @@
       <c r="F136" s="8"/>
       <c r="G136" s="10"/>
     </row>
-    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A137" s="4" t="s">
         <v>259</v>
       </c>
@@ -14370,7 +14452,7 @@
       </c>
       <c r="G137" s="9"/>
     </row>
-    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A138" s="8" t="s">
         <v>261</v>
       </c>
@@ -14391,7 +14473,7 @@
       </c>
       <c r="G138" s="10"/>
     </row>
-    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A139" s="4" t="s">
         <v>263</v>
       </c>
@@ -14412,7 +14494,7 @@
       </c>
       <c r="G139" s="9"/>
     </row>
-    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A140" s="8" t="s">
         <v>265</v>
       </c>
@@ -14425,7 +14507,7 @@
       <c r="F140" s="8"/>
       <c r="G140" s="10"/>
     </row>
-    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A141" s="4" t="s">
         <v>267</v>
       </c>
@@ -14438,7 +14520,7 @@
       <c r="F141" s="4"/>
       <c r="G141" s="9"/>
     </row>
-    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="8" t="s">
         <v>269</v>
       </c>
@@ -14455,7 +14537,7 @@
       </c>
       <c r="G142" s="10"/>
     </row>
-    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A143" s="4" t="s">
         <v>271</v>
       </c>
@@ -14468,7 +14550,7 @@
       <c r="F143" s="4"/>
       <c r="G143" s="9"/>
     </row>
-    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A144" s="8" t="s">
         <v>273</v>
       </c>
@@ -14485,7 +14567,7 @@
       </c>
       <c r="G144" s="10"/>
     </row>
-    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A145" s="4" t="s">
         <v>275</v>
       </c>
@@ -14498,7 +14580,7 @@
       <c r="F145" s="4"/>
       <c r="G145" s="9"/>
     </row>
-    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A146" s="8" t="s">
         <v>277</v>
       </c>
@@ -14511,7 +14593,7 @@
       <c r="F146" s="8"/>
       <c r="G146" s="10"/>
     </row>
-    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A147" s="4" t="s">
         <v>279</v>
       </c>
@@ -14522,7 +14604,7 @@
       <c r="F147" s="4"/>
       <c r="G147" s="9"/>
     </row>
-    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A148" s="8" t="s">
         <v>281</v>
       </c>
@@ -14535,7 +14617,7 @@
       <c r="F148" s="8"/>
       <c r="G148" s="10"/>
     </row>
-    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A149" s="4" t="s">
         <v>283</v>
       </c>
@@ -14548,7 +14630,7 @@
       <c r="F149" s="4"/>
       <c r="G149" s="9"/>
     </row>
-    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A150" s="8" t="s">
         <v>285</v>
       </c>
@@ -14561,7 +14643,7 @@
       <c r="F150" s="8"/>
       <c r="G150" s="10"/>
     </row>
-    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A151" s="4" t="s">
         <v>287</v>
       </c>
@@ -14574,7 +14656,7 @@
       <c r="F151" s="4"/>
       <c r="G151" s="9"/>
     </row>
-    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A152" s="8" t="s">
         <v>289</v>
       </c>
@@ -14600,7 +14682,7 @@
       <c r="F153" s="4"/>
       <c r="G153" s="9"/>
     </row>
-    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A154" s="8" t="s">
         <v>293</v>
       </c>
@@ -14619,7 +14701,7 @@
       </c>
       <c r="G154" s="10"/>
     </row>
-    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A155" s="4" t="s">
         <v>295</v>
       </c>
@@ -14632,7 +14714,7 @@
       <c r="F155" s="4"/>
       <c r="G155" s="9"/>
     </row>
-    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A156" s="8" t="s">
         <v>297</v>
       </c>
@@ -14645,7 +14727,7 @@
       <c r="F156" s="8"/>
       <c r="G156" s="10"/>
     </row>
-    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A157" s="4" t="s">
         <v>299</v>
       </c>
@@ -14658,7 +14740,7 @@
       <c r="F157" s="4"/>
       <c r="G157" s="9"/>
     </row>
-    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A158" s="8" t="s">
         <v>301</v>
       </c>
@@ -14671,7 +14753,7 @@
       <c r="F158" s="8"/>
       <c r="G158" s="10"/>
     </row>
-    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A159" s="4" t="s">
         <v>303</v>
       </c>
@@ -14684,7 +14766,7 @@
       <c r="F159" s="4"/>
       <c r="G159" s="9"/>
     </row>
-    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A160" s="8" t="s">
         <v>305</v>
       </c>
@@ -14697,7 +14779,7 @@
       <c r="F160" s="8"/>
       <c r="G160" s="10"/>
     </row>
-    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A161" s="4" t="s">
         <v>307</v>
       </c>
@@ -14710,7 +14792,7 @@
       <c r="F161" s="4"/>
       <c r="G161" s="9"/>
     </row>
-    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A162" s="8" t="s">
         <v>309</v>
       </c>
@@ -14723,7 +14805,7 @@
       <c r="F162" s="8"/>
       <c r="G162" s="10"/>
     </row>
-    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A163" s="4" t="s">
         <v>311</v>
       </c>
@@ -14736,7 +14818,7 @@
       <c r="F163" s="4"/>
       <c r="G163" s="9"/>
     </row>
-    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A164" s="8" t="s">
         <v>313</v>
       </c>
@@ -14749,7 +14831,7 @@
       <c r="F164" s="8"/>
       <c r="G164" s="10"/>
     </row>
-    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A165" s="4" t="s">
         <v>315</v>
       </c>
@@ -14762,7 +14844,7 @@
       <c r="F165" s="4"/>
       <c r="G165" s="9"/>
     </row>
-    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A166" s="8" t="s">
         <v>317</v>
       </c>
@@ -14775,7 +14857,7 @@
       <c r="F166" s="8"/>
       <c r="G166" s="10"/>
     </row>
-    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A167" s="4" t="s">
         <v>319</v>
       </c>
@@ -14796,7 +14878,7 @@
       </c>
       <c r="G167" s="9"/>
     </row>
-    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A168" s="8" t="s">
         <v>321</v>
       </c>
@@ -14809,7 +14891,7 @@
       <c r="F168" s="8"/>
       <c r="G168" s="10"/>
     </row>
-    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A169" s="4" t="s">
         <v>323</v>
       </c>
@@ -14822,7 +14904,7 @@
       <c r="F169" s="4"/>
       <c r="G169" s="9"/>
     </row>
-    <row r="170" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="170" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A170" s="8" t="s">
         <v>325</v>
       </c>
@@ -14836,40 +14918,7 @@
       <c r="G170" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:G170" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="CAÇAMBA IVECO 28260 PL PIG 5304 POTY"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS  SR004989 PLACA SLT 6C49"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS R002697 PLACA SLT 6D33"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR002618 PLACA SLT 6D30"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR002652 PLACA SLT 6D34"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR002658 PLACA SLT 6D25"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR004619 PLACA SLT 6C45"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR005043 PLACA SLT 6C48"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR005574 PLACA SLT 6C43"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR005579 PLACA SLT 6C50"/>
-        <filter val="CAÇAMBA NOVA VW 26260 CHASSIS SR005705 PLACA SLT 6C44"/>
-        <filter val="CAÇAMBA NOVA VW 26330 Chassi: 9536C8TD8RR058330 | DANFE 618388 SLR 6C65"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058361 PLACA SLR-0E27"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058408 PLACA SLR-4G15"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058635 PLACA SLR-4G25"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058697 PLACA SLR-4E18"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058778 PLACA SLR-4G29"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR058862 PLACA SLR-0i11"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR059087 PLACA SLR-0E23"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSIS RR059154 PLACA SLR-0E26"/>
-        <filter val="CAÇAMBA NOVA VW 26330 CHSSISRR058957 PLACA SLR-0E19"/>
-        <filter val="CAÇAMBA SCANEA 310 PL PIN 0144 POTY"/>
-        <filter val="CAÇAMBA VOLKS 24260 PL QRR 5B87 POTY"/>
-        <filter val="CAÇAMBA VOLKS 24260 PL QRR 8A07 POTY"/>
-        <filter val="CAÇAMBA VOLVO 270 PL PIZ 3804 POTY"/>
-        <filter val="CAÇAMBA VOLVO 270 PL PIZ 3i14 POTY"/>
-        <filter val="CAÇAMBA VOLVO 330 PL QRR 4G34 POTY"/>
-        <filter val="CAÇAMBÃO COLOM  PLACA PIA 7B52"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A6:G170" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G3"/>
     <mergeCell ref="A5:G5"/>
@@ -16238,7 +16287,7 @@
       <c r="G88" s="10"/>
     </row>
     <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A89" s="15" t="s">
+      <c r="A89" s="4" t="s">
         <v>163</v>
       </c>
       <c r="B89" s="4" t="s">
@@ -17568,6 +17617,2954 @@
         <v>326</v>
       </c>
       <c r="C170" s="8"/>
+      <c r="D170" s="8"/>
+      <c r="E170" s="8"/>
+      <c r="F170" s="8"/>
+      <c r="G170" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G170" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACAF762F-0246-4430-BED4-831A0A8E9DEF}">
+  <dimension ref="A1:G170"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
+        <v>417</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G32" s="10"/>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F54" s="8"/>
+      <c r="G54" s="10"/>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F56" s="8"/>
+      <c r="G56" s="10"/>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F57" s="4"/>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F58" s="8"/>
+      <c r="G58" s="10"/>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F59" s="4"/>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G60" s="10"/>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10"/>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G67" s="9"/>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8"/>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10"/>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8"/>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F85" s="4"/>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F86" s="8"/>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F87" s="4"/>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F88" s="8"/>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F90" s="8"/>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F91" s="4"/>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F92" s="8"/>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F93" s="4"/>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F94" s="8"/>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+      <c r="F95" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G95" s="9"/>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="8"/>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8"/>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8"/>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+      <c r="F105" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8"/>
+      <c r="F106" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8"/>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="C112" s="8"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="8"/>
+      <c r="G112" s="10"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E113" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="9"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C114" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D114" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F114" s="8"/>
+      <c r="G114" s="10"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D115" s="4"/>
+      <c r="E115" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F115" s="4"/>
+      <c r="G115" s="9"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C116" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D116" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F116" s="8"/>
+      <c r="G116" s="10"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D117" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E117" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F117" s="4"/>
+      <c r="G117" s="9"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B118" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C118" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D118" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F118" s="8"/>
+      <c r="G118" s="10"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D119" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E119" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F119" s="4"/>
+      <c r="G119" s="9"/>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C120" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D120" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F120" s="8"/>
+      <c r="G120" s="10"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D121" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E121" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F121" s="4"/>
+      <c r="G121" s="9"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B122" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C122" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E122" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="F122" s="8"/>
+      <c r="G122" s="10"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E123" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F123" s="4"/>
+      <c r="G123" s="9"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B124" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C124" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D124" s="8"/>
+      <c r="E124" s="8"/>
+      <c r="F124" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G124" s="10"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D125" s="4"/>
+      <c r="E125" s="4"/>
+      <c r="F125" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G125" s="9"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C126" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D126" s="8"/>
+      <c r="E126" s="8"/>
+      <c r="F126" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="G126" s="10"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E127" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G127" s="9"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C128" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="8"/>
+      <c r="E128" s="8"/>
+      <c r="F128" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G128" s="10"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="4"/>
+      <c r="E129" s="4"/>
+      <c r="F129" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G129" s="9"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="8"/>
+      <c r="E130" s="8"/>
+      <c r="F130" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G130" s="10"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G131" s="9"/>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D132" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F132" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D133" s="4"/>
+      <c r="E133" s="4"/>
+      <c r="F133" s="4"/>
+      <c r="G133" s="9"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C134" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D134" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F134" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="10"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E135" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G135" s="9"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C136" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D136" s="8"/>
+      <c r="E136" s="8"/>
+      <c r="F136" s="8"/>
+      <c r="G136" s="10"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E137" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="9"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C138" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D138" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F138" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="10"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D139" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E139" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G139" s="9"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C140" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D140" s="8"/>
+      <c r="E140" s="8"/>
+      <c r="F140" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="G140" s="10"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D141" s="4"/>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G141" s="9"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C142" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="8"/>
+      <c r="E142" s="8"/>
+      <c r="F142" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G142" s="10"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G143" s="9"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="8"/>
+      <c r="E144" s="8"/>
+      <c r="F144" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G144" s="10"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D145" s="4"/>
+      <c r="E145" s="4"/>
+      <c r="F145" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G145" s="9"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B146" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C146" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G146" s="10"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C147" s="15" t="s">
+        <v>373</v>
+      </c>
+      <c r="E147" s="4"/>
+      <c r="F147" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G147" s="9"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B148" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C148" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D148" s="8"/>
+      <c r="E148" s="8"/>
+      <c r="F148" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G148" s="10"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C149" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D149" s="4"/>
+      <c r="E149" s="4"/>
+      <c r="F149" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G149" s="9"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C150" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D150" s="8"/>
+      <c r="E150" s="8"/>
+      <c r="F150" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G150" s="10"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C151" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G151" s="9"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B152" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C152" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
+      <c r="F152" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G152" s="10"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C153" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D153" s="4"/>
+      <c r="E153" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F153" s="4"/>
+      <c r="G153" s="9"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C154" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D154" s="8"/>
+      <c r="E154" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F154" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="10"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C155" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G155" s="9"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C156" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8"/>
+      <c r="F156" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G156" s="10"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C157" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G157" s="9"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B158" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C158" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8"/>
+      <c r="F158" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G158" s="10"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="9"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B160" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C160" s="8"/>
+      <c r="D160" s="8"/>
+      <c r="E160" s="8"/>
+      <c r="F160" s="8"/>
+      <c r="G160" s="10"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+      <c r="G161" s="9"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B162" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C162" s="8"/>
+      <c r="D162" s="8"/>
+      <c r="E162" s="8"/>
+      <c r="F162" s="8"/>
+      <c r="G162" s="10"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+      <c r="G163" s="9"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B164" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C164" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D164" s="8"/>
+      <c r="E164" s="8"/>
+      <c r="F164" s="8"/>
+      <c r="G164" s="10"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C165" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D165" s="4"/>
+      <c r="E165" s="4"/>
+      <c r="F165" s="4"/>
+      <c r="G165" s="9"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B166" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C166" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D166" s="8"/>
+      <c r="E166" s="8"/>
+      <c r="F166" s="8"/>
+      <c r="G166" s="10"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D167" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E167" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G167" s="9"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B168" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C168" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D168" s="8"/>
+      <c r="E168" s="8"/>
+      <c r="F168" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G168" s="10"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C169" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G169" s="9"/>
+    </row>
+    <row r="170" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A170" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B170" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C170" s="8" t="s">
+        <v>424</v>
+      </c>
       <c r="D170" s="8"/>
       <c r="E170" s="8"/>
       <c r="F170" s="8"/>

</xml_diff>

<commit_message>
FECHAMENTO FEVEREIRO: ATIVOS INCIO 6 E 8 LANÇADOS:19/03 17:10H
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E09335-069C-480F-9703-F0893F7097BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB31D9BC-2B66-451B-9548-F76F2690E4DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3755" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3876" uniqueCount="429">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1326,6 +1326,18 @@
   </si>
   <si>
     <t>DEVOLVIDA</t>
+  </si>
+  <si>
+    <t>NAYRON - PCM / UC</t>
+  </si>
+  <si>
+    <t>LUCIANO - OFICINA</t>
+  </si>
+  <si>
+    <t>PARADA NA OFICINA</t>
+  </si>
+  <si>
+    <t>SAMUEL - TRANSPORTE / UC</t>
   </si>
 </sst>
 </file>
@@ -1513,13 +1525,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
@@ -2252,45 +2264,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="15" t="s">
         <v>338</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -4638,45 +4650,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="15" t="s">
         <v>365</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -7018,45 +7030,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="15" t="s">
         <v>385</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -9666,45 +9678,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="15" t="s">
         <v>408</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -12316,45 +12328,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="15" t="s">
         <v>411</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -14945,45 +14957,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="15" t="s">
         <v>416</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -17650,45 +17662,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="15" t="s">
         <v>417</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
@@ -17724,7 +17736,9 @@
         <v>373</v>
       </c>
       <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F7" s="4" t="s">
         <v>371</v>
       </c>
@@ -17756,7 +17770,9 @@
         <v>373</v>
       </c>
       <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F9" s="4" t="s">
         <v>371</v>
       </c>
@@ -17773,7 +17789,9 @@
         <v>373</v>
       </c>
       <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F10" s="8" t="s">
         <v>371</v>
       </c>
@@ -17820,7 +17838,9 @@
         <v>373</v>
       </c>
       <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F13" s="4" t="s">
         <v>371</v>
       </c>
@@ -17837,7 +17857,9 @@
         <v>373</v>
       </c>
       <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F14" s="8" t="s">
         <v>371</v>
       </c>
@@ -17854,7 +17876,9 @@
         <v>373</v>
       </c>
       <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
+      <c r="E15" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F15" s="4" t="s">
         <v>371</v>
       </c>
@@ -17886,7 +17910,9 @@
         <v>373</v>
       </c>
       <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F17" s="4" t="s">
         <v>371</v>
       </c>
@@ -17903,7 +17929,9 @@
         <v>373</v>
       </c>
       <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
+      <c r="E18" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F18" s="8" t="s">
         <v>371</v>
       </c>
@@ -17920,7 +17948,9 @@
         <v>373</v>
       </c>
       <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F19" s="4" t="s">
         <v>371</v>
       </c>
@@ -17937,7 +17967,9 @@
         <v>373</v>
       </c>
       <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
+      <c r="E20" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F20" s="8" t="s">
         <v>333</v>
       </c>
@@ -17969,7 +18001,9 @@
         <v>373</v>
       </c>
       <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
+      <c r="E22" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F22" s="8" t="s">
         <v>371</v>
       </c>
@@ -18007,7 +18041,9 @@
         <v>373</v>
       </c>
       <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
+      <c r="E24" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F24" s="8" t="s">
         <v>333</v>
       </c>
@@ -18024,7 +18060,9 @@
         <v>373</v>
       </c>
       <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
+      <c r="E25" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F25" s="4" t="s">
         <v>371</v>
       </c>
@@ -18041,7 +18079,9 @@
         <v>373</v>
       </c>
       <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
+      <c r="E26" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F26" s="8" t="s">
         <v>371</v>
       </c>
@@ -18058,7 +18098,9 @@
         <v>373</v>
       </c>
       <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F27" s="4" t="s">
         <v>371</v>
       </c>
@@ -18096,7 +18138,9 @@
         <v>373</v>
       </c>
       <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F29" s="4" t="s">
         <v>333</v>
       </c>
@@ -18113,7 +18157,9 @@
         <v>373</v>
       </c>
       <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
+      <c r="E30" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F30" s="8" t="s">
         <v>333</v>
       </c>
@@ -18130,7 +18176,9 @@
         <v>373</v>
       </c>
       <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F31" s="4" t="s">
         <v>371</v>
       </c>
@@ -18147,11 +18195,15 @@
         <v>373</v>
       </c>
       <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
+      <c r="E32" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F32" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="G32" s="10"/>
+      <c r="G32" s="10" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A33" s="4" t="s">
@@ -18164,7 +18216,9 @@
         <v>418</v>
       </c>
       <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
+      <c r="E33" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F33" s="4" t="s">
         <v>333</v>
       </c>
@@ -18177,10 +18231,16 @@
       <c r="B34" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C34" s="8"/>
+      <c r="C34" s="8" t="s">
+        <v>419</v>
+      </c>
       <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
+      <c r="E34" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G34" s="10"/>
     </row>
     <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
@@ -18217,7 +18277,9 @@
         <v>373</v>
       </c>
       <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
+      <c r="E36" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F36" s="8" t="s">
         <v>333</v>
       </c>
@@ -18234,7 +18296,9 @@
         <v>372</v>
       </c>
       <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="E37" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F37" s="4" t="s">
         <v>333</v>
       </c>
@@ -18251,7 +18315,9 @@
         <v>373</v>
       </c>
       <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
+      <c r="E38" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F38" s="8" t="s">
         <v>333</v>
       </c>
@@ -18268,7 +18334,9 @@
         <v>373</v>
       </c>
       <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="E39" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F39" s="4" t="s">
         <v>333</v>
       </c>
@@ -18298,7 +18366,9 @@
         <v>373</v>
       </c>
       <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
+      <c r="E41" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F41" s="4" t="s">
         <v>333</v>
       </c>
@@ -18315,7 +18385,9 @@
         <v>372</v>
       </c>
       <c r="D42" s="8"/>
-      <c r="E42" s="8"/>
+      <c r="E42" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F42" s="8" t="s">
         <v>333</v>
       </c>
@@ -18332,7 +18404,9 @@
         <v>372</v>
       </c>
       <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
+      <c r="E43" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F43" s="4" t="s">
         <v>333</v>
       </c>
@@ -18349,7 +18423,9 @@
         <v>373</v>
       </c>
       <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
+      <c r="E44" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F44" s="8" t="s">
         <v>371</v>
       </c>
@@ -18366,7 +18442,9 @@
         <v>372</v>
       </c>
       <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
+      <c r="E45" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F45" s="4" t="s">
         <v>333</v>
       </c>
@@ -18402,7 +18480,9 @@
         <v>373</v>
       </c>
       <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
+      <c r="E47" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F47" s="4" t="s">
         <v>371</v>
       </c>
@@ -18419,7 +18499,9 @@
         <v>373</v>
       </c>
       <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
+      <c r="E48" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F48" s="8" t="s">
         <v>333</v>
       </c>
@@ -18436,7 +18518,9 @@
         <v>373</v>
       </c>
       <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
+      <c r="E49" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F49" s="4" t="s">
         <v>333</v>
       </c>
@@ -18453,7 +18537,9 @@
         <v>372</v>
       </c>
       <c r="D50" s="8"/>
-      <c r="E50" s="8"/>
+      <c r="E50" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F50" s="8" t="s">
         <v>333</v>
       </c>
@@ -18487,7 +18573,9 @@
         <v>372</v>
       </c>
       <c r="D52" s="8"/>
-      <c r="E52" s="8"/>
+      <c r="E52" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F52" s="8" t="s">
         <v>333</v>
       </c>
@@ -18526,10 +18614,14 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F54" s="8"/>
-      <c r="G54" s="10"/>
+        <v>428</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G54" s="10" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A55" s="4" t="s">
@@ -18564,10 +18656,14 @@
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F56" s="8"/>
-      <c r="G56" s="10"/>
+        <v>428</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G56" s="10" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A57" s="4" t="s">
@@ -18581,9 +18677,11 @@
       </c>
       <c r="D57" s="4"/>
       <c r="E57" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F57" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G57" s="9"/>
     </row>
     <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -18598,10 +18696,14 @@
       </c>
       <c r="D58" s="8"/>
       <c r="E58" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F58" s="8"/>
-      <c r="G58" s="10"/>
+        <v>428</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A59" s="4" t="s">
@@ -18617,9 +18719,11 @@
         <v>405</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F59" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G59" s="9"/>
     </row>
     <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -18633,11 +18737,15 @@
         <v>373</v>
       </c>
       <c r="D60" s="8"/>
-      <c r="E60" s="8"/>
+      <c r="E60" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F60" s="8" t="s">
         <v>333</v>
       </c>
-      <c r="G60" s="10"/>
+      <c r="G60" s="10" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A61" s="4" t="s">
@@ -18650,7 +18758,9 @@
         <v>419</v>
       </c>
       <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
+      <c r="E61" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F61" s="4" t="s">
         <v>333</v>
       </c>
@@ -18699,11 +18809,15 @@
         <v>373</v>
       </c>
       <c r="D64" s="8"/>
-      <c r="E64" s="8"/>
+      <c r="E64" s="8" t="s">
+        <v>426</v>
+      </c>
       <c r="F64" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="G64" s="10"/>
+      <c r="G64" s="10" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A65" s="4" t="s">
@@ -18716,7 +18830,9 @@
         <v>373</v>
       </c>
       <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
+      <c r="E65" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F65" s="4" t="s">
         <v>371</v>
       </c>
@@ -18754,7 +18870,9 @@
         <v>372</v>
       </c>
       <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
+      <c r="E67" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F67" s="4" t="s">
         <v>333</v>
       </c>
@@ -18771,7 +18889,9 @@
         <v>373</v>
       </c>
       <c r="D68" s="8"/>
-      <c r="E68" s="8"/>
+      <c r="E68" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F68" s="8" t="s">
         <v>371</v>
       </c>
@@ -18788,7 +18908,9 @@
         <v>373</v>
       </c>
       <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
+      <c r="E69" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F69" s="4" t="s">
         <v>371</v>
       </c>
@@ -18805,7 +18927,9 @@
         <v>373</v>
       </c>
       <c r="D70" s="8"/>
-      <c r="E70" s="8"/>
+      <c r="E70" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F70" s="8" t="s">
         <v>371</v>
       </c>
@@ -18822,7 +18946,9 @@
         <v>377</v>
       </c>
       <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
+      <c r="E71" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F71" s="4" t="s">
         <v>371</v>
       </c>
@@ -18856,7 +18982,9 @@
         <v>373</v>
       </c>
       <c r="D73" s="4"/>
-      <c r="E73" s="4"/>
+      <c r="E73" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F73" s="4" t="s">
         <v>333</v>
       </c>
@@ -18894,7 +19022,9 @@
         <v>373</v>
       </c>
       <c r="D75" s="4"/>
-      <c r="E75" s="4"/>
+      <c r="E75" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F75" s="4" t="s">
         <v>333</v>
       </c>
@@ -18911,7 +19041,9 @@
         <v>384</v>
       </c>
       <c r="D76" s="8"/>
-      <c r="E76" s="8"/>
+      <c r="E76" s="8" t="s">
+        <v>426</v>
+      </c>
       <c r="F76" s="8" t="s">
         <v>333</v>
       </c>
@@ -18928,7 +19060,9 @@
         <v>376</v>
       </c>
       <c r="D77" s="4"/>
-      <c r="E77" s="4"/>
+      <c r="E77" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F77" s="4" t="s">
         <v>333</v>
       </c>
@@ -18945,7 +19079,9 @@
         <v>373</v>
       </c>
       <c r="D78" s="8"/>
-      <c r="E78" s="8"/>
+      <c r="E78" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F78" s="8" t="s">
         <v>371</v>
       </c>
@@ -18981,11 +19117,15 @@
         <v>373</v>
       </c>
       <c r="D80" s="8"/>
-      <c r="E80" s="8"/>
+      <c r="E80" s="8" t="s">
+        <v>426</v>
+      </c>
       <c r="F80" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="G80" s="10"/>
+      <c r="G80" s="10" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A81" s="4" t="s">
@@ -18998,7 +19138,9 @@
         <v>372</v>
       </c>
       <c r="D81" s="4"/>
-      <c r="E81" s="4"/>
+      <c r="E81" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F81" s="4" t="s">
         <v>333</v>
       </c>
@@ -19015,7 +19157,9 @@
         <v>420</v>
       </c>
       <c r="D82" s="8"/>
-      <c r="E82" s="8"/>
+      <c r="E82" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F82" s="8"/>
       <c r="G82" s="10"/>
     </row>
@@ -19030,7 +19174,9 @@
         <v>384</v>
       </c>
       <c r="D83" s="4"/>
-      <c r="E83" s="4"/>
+      <c r="E83" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F83" s="4"/>
       <c r="G83" s="9"/>
     </row>
@@ -19065,9 +19211,11 @@
         <v>391</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F85" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G85" s="9"/>
     </row>
     <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19084,9 +19232,11 @@
         <v>388</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F86" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G86" s="10"/>
     </row>
     <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19103,9 +19253,11 @@
         <v>400</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F87" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G87" s="9"/>
     </row>
     <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19122,9 +19274,11 @@
         <v>407</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F88" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F88" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G88" s="10"/>
     </row>
     <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19162,9 +19316,11 @@
         <v>402</v>
       </c>
       <c r="E90" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F90" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G90" s="10"/>
     </row>
     <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19181,9 +19337,11 @@
         <v>394</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F91" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G91" s="9"/>
     </row>
     <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19200,9 +19358,11 @@
         <v>399</v>
       </c>
       <c r="E92" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F92" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G92" s="10"/>
     </row>
     <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19219,9 +19379,11 @@
         <v>393</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F93" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G93" s="9"/>
     </row>
     <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19236,9 +19398,11 @@
       </c>
       <c r="D94" s="8"/>
       <c r="E94" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F94" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G94" s="10"/>
     </row>
     <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19252,11 +19416,15 @@
         <v>373</v>
       </c>
       <c r="D95" s="4"/>
-      <c r="E95" s="4"/>
+      <c r="E95" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F95" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="G95" s="9"/>
+      <c r="G95" s="9" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="8" t="s">
@@ -19318,7 +19486,9 @@
         <v>373</v>
       </c>
       <c r="D99" s="4"/>
-      <c r="E99" s="4"/>
+      <c r="E99" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F99" s="4" t="s">
         <v>333</v>
       </c>
@@ -19394,7 +19564,9 @@
         <v>373</v>
       </c>
       <c r="D103" s="4"/>
-      <c r="E103" s="4"/>
+      <c r="E103" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F103" s="4" t="s">
         <v>371</v>
       </c>
@@ -19426,7 +19598,9 @@
         <v>373</v>
       </c>
       <c r="D105" s="4"/>
-      <c r="E105" s="4"/>
+      <c r="E105" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F105" s="4" t="s">
         <v>333</v>
       </c>
@@ -19443,7 +19617,9 @@
         <v>373</v>
       </c>
       <c r="D106" s="8"/>
-      <c r="E106" s="8"/>
+      <c r="E106" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F106" s="8" t="s">
         <v>421</v>
       </c>
@@ -19508,9 +19684,7 @@
       <c r="F109" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="G109" s="9" t="s">
-        <v>354</v>
-      </c>
+      <c r="G109" s="9"/>
     </row>
     <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="8" t="s">
@@ -19594,9 +19768,11 @@
         <v>406</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F114" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F114" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G114" s="10"/>
     </row>
     <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19611,9 +19787,11 @@
       </c>
       <c r="D115" s="4"/>
       <c r="E115" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F115" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F115" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G115" s="9"/>
     </row>
     <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19630,9 +19808,11 @@
         <v>397</v>
       </c>
       <c r="E116" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F116" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F116" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G116" s="10"/>
     </row>
     <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19649,9 +19829,11 @@
         <v>395</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F117" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F117" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G117" s="9"/>
     </row>
     <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19668,9 +19850,11 @@
         <v>404</v>
       </c>
       <c r="E118" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F118" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F118" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G118" s="10"/>
     </row>
     <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19687,9 +19871,11 @@
         <v>401</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F119" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G119" s="9"/>
     </row>
     <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19706,10 +19892,14 @@
         <v>396</v>
       </c>
       <c r="E120" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F120" s="8"/>
-      <c r="G120" s="10"/>
+        <v>428</v>
+      </c>
+      <c r="F120" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G120" s="10" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="4" t="s">
@@ -19725,9 +19915,11 @@
         <v>390</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F121" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F121" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G121" s="9"/>
     </row>
     <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19744,9 +19936,11 @@
         <v>389</v>
       </c>
       <c r="E122" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="F122" s="8"/>
+        <v>428</v>
+      </c>
+      <c r="F122" s="8" t="s">
+        <v>333</v>
+      </c>
       <c r="G122" s="10"/>
     </row>
     <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19763,9 +19957,11 @@
         <v>403</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F123" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F123" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G123" s="9"/>
     </row>
     <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19779,7 +19975,9 @@
         <v>375</v>
       </c>
       <c r="D124" s="8"/>
-      <c r="E124" s="8"/>
+      <c r="E124" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F124" s="8" t="s">
         <v>333</v>
       </c>
@@ -19813,7 +20011,9 @@
         <v>373</v>
       </c>
       <c r="D126" s="8"/>
-      <c r="E126" s="8"/>
+      <c r="E126" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F126" s="8" t="s">
         <v>422</v>
       </c>
@@ -19851,7 +20051,9 @@
         <v>373</v>
       </c>
       <c r="D128" s="8"/>
-      <c r="E128" s="8"/>
+      <c r="E128" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F128" s="8" t="s">
         <v>371</v>
       </c>
@@ -19885,7 +20087,9 @@
         <v>373</v>
       </c>
       <c r="D130" s="8"/>
-      <c r="E130" s="8"/>
+      <c r="E130" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F130" s="8" t="s">
         <v>371</v>
       </c>
@@ -19902,7 +20106,9 @@
         <v>373</v>
       </c>
       <c r="D131" s="4"/>
-      <c r="E131" s="4"/>
+      <c r="E131" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F131" s="4" t="s">
         <v>333</v>
       </c>
@@ -20077,7 +20283,9 @@
         <v>373</v>
       </c>
       <c r="D140" s="8"/>
-      <c r="E140" s="8"/>
+      <c r="E140" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F140" s="8" t="s">
         <v>423</v>
       </c>
@@ -20094,7 +20302,9 @@
         <v>373</v>
       </c>
       <c r="D141" s="4"/>
-      <c r="E141" s="4"/>
+      <c r="E141" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F141" s="4" t="s">
         <v>333</v>
       </c>
@@ -20111,7 +20321,9 @@
         <v>373</v>
       </c>
       <c r="D142" s="8"/>
-      <c r="E142" s="8"/>
+      <c r="E142" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F142" s="8" t="s">
         <v>371</v>
       </c>
@@ -20128,7 +20340,9 @@
         <v>373</v>
       </c>
       <c r="D143" s="4"/>
-      <c r="E143" s="4"/>
+      <c r="E143" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F143" s="4" t="s">
         <v>333</v>
       </c>
@@ -20145,7 +20359,9 @@
         <v>373</v>
       </c>
       <c r="D144" s="8"/>
-      <c r="E144" s="8"/>
+      <c r="E144" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F144" s="8" t="s">
         <v>371</v>
       </c>
@@ -20162,7 +20378,9 @@
         <v>373</v>
       </c>
       <c r="D145" s="4"/>
-      <c r="E145" s="4"/>
+      <c r="E145" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F145" s="4" t="s">
         <v>333</v>
       </c>
@@ -20179,7 +20397,9 @@
         <v>373</v>
       </c>
       <c r="D146" s="8"/>
-      <c r="E146" s="8"/>
+      <c r="E146" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F146" s="8" t="s">
         <v>333</v>
       </c>
@@ -20192,10 +20412,12 @@
       <c r="B147" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="C147" s="15" t="s">
-        <v>373</v>
-      </c>
-      <c r="E147" s="4"/>
+      <c r="C147" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="E147" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F147" s="4" t="s">
         <v>333</v>
       </c>
@@ -20212,7 +20434,9 @@
         <v>373</v>
       </c>
       <c r="D148" s="8"/>
-      <c r="E148" s="8"/>
+      <c r="E148" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F148" s="8" t="s">
         <v>333</v>
       </c>
@@ -20229,7 +20453,9 @@
         <v>373</v>
       </c>
       <c r="D149" s="4"/>
-      <c r="E149" s="4"/>
+      <c r="E149" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F149" s="4" t="s">
         <v>333</v>
       </c>
@@ -20246,7 +20472,9 @@
         <v>373</v>
       </c>
       <c r="D150" s="8"/>
-      <c r="E150" s="8"/>
+      <c r="E150" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F150" s="8" t="s">
         <v>333</v>
       </c>
@@ -20263,7 +20491,9 @@
         <v>373</v>
       </c>
       <c r="D151" s="4"/>
-      <c r="E151" s="4"/>
+      <c r="E151" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F151" s="4" t="s">
         <v>333</v>
       </c>
@@ -20280,7 +20510,9 @@
         <v>373</v>
       </c>
       <c r="D152" s="8"/>
-      <c r="E152" s="8"/>
+      <c r="E152" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F152" s="8" t="s">
         <v>333</v>
       </c>
@@ -20298,9 +20530,11 @@
       </c>
       <c r="D153" s="4"/>
       <c r="E153" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="F153" s="4"/>
+        <v>428</v>
+      </c>
+      <c r="F153" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="G153" s="9"/>
     </row>
     <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -20333,7 +20567,9 @@
         <v>373</v>
       </c>
       <c r="D155" s="4"/>
-      <c r="E155" s="4"/>
+      <c r="E155" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F155" s="4" t="s">
         <v>333</v>
       </c>
@@ -20350,7 +20586,9 @@
         <v>376</v>
       </c>
       <c r="D156" s="8"/>
-      <c r="E156" s="8"/>
+      <c r="E156" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F156" s="8" t="s">
         <v>333</v>
       </c>
@@ -20367,7 +20605,9 @@
         <v>384</v>
       </c>
       <c r="D157" s="4"/>
-      <c r="E157" s="4"/>
+      <c r="E157" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F157" s="4" t="s">
         <v>333</v>
       </c>
@@ -20384,7 +20624,9 @@
         <v>376</v>
       </c>
       <c r="D158" s="8"/>
-      <c r="E158" s="8"/>
+      <c r="E158" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F158" s="8" t="s">
         <v>333</v>
       </c>
@@ -20466,7 +20708,9 @@
         <v>372</v>
       </c>
       <c r="D164" s="8"/>
-      <c r="E164" s="8"/>
+      <c r="E164" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F164" s="8"/>
       <c r="G164" s="10"/>
     </row>
@@ -20481,7 +20725,9 @@
         <v>372</v>
       </c>
       <c r="D165" s="4"/>
-      <c r="E165" s="4"/>
+      <c r="E165" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F165" s="4"/>
       <c r="G165" s="9"/>
     </row>
@@ -20496,7 +20742,9 @@
         <v>372</v>
       </c>
       <c r="D166" s="8"/>
-      <c r="E166" s="8"/>
+      <c r="E166" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F166" s="8"/>
       <c r="G166" s="10"/>
     </row>
@@ -20514,10 +20762,10 @@
         <v>358</v>
       </c>
       <c r="E167" s="4" t="s">
-        <v>356</v>
+        <v>425</v>
       </c>
       <c r="F167" s="4" t="s">
-        <v>333</v>
+        <v>371</v>
       </c>
       <c r="G167" s="9"/>
     </row>
@@ -20532,7 +20780,9 @@
         <v>373</v>
       </c>
       <c r="D168" s="8"/>
-      <c r="E168" s="8"/>
+      <c r="E168" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F168" s="8" t="s">
         <v>371</v>
       </c>
@@ -20549,7 +20799,9 @@
         <v>373</v>
       </c>
       <c r="D169" s="4"/>
-      <c r="E169" s="4"/>
+      <c r="E169" s="4" t="s">
+        <v>425</v>
+      </c>
       <c r="F169" s="4" t="s">
         <v>371</v>
       </c>
@@ -20566,7 +20818,9 @@
         <v>424</v>
       </c>
       <c r="D170" s="8"/>
-      <c r="E170" s="8"/>
+      <c r="E170" s="8" t="s">
+        <v>425</v>
+      </c>
       <c r="F170" s="8"/>
       <c r="G170" s="10"/>
     </row>

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA FROTA POTY: 20/03 13:140H
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF835BC-A7B5-4CC6-A12B-FEEEBD601BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CC06A0F-459B-49D2-865D-C95B7C07FB14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'19'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'20'!$A$6:$G$170</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3876" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3883" uniqueCount="433">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1304,9 +1304,6 @@
     <t>DATA DA CONFERENCIA: 19/03/2026</t>
   </si>
   <si>
-    <t>DATA DA CONFERENCIA: 20/03/2026</t>
-  </si>
-  <si>
     <t>FORTALEZA</t>
   </si>
   <si>
@@ -1338,6 +1335,21 @@
   </si>
   <si>
     <t>SAMUEL - TRANSPORTE / UC</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERÊNCIA: 20/03/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jardel Ferreira Santos </t>
+  </si>
+  <si>
+    <t>transito de Cadoz para Teresina 20/03/2026</t>
+  </si>
+  <si>
+    <t>TRANSITO: CADOZ X TERESINA</t>
+  </si>
+  <si>
+    <t>REGENERAÇÃO</t>
   </si>
 </sst>
 </file>
@@ -1491,7 +1503,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1531,6 +1543,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -17693,7 +17708,7 @@
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
-        <v>417</v>
+        <v>428</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
@@ -17737,7 +17752,7 @@
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>371</v>
@@ -17771,7 +17786,7 @@
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>371</v>
@@ -17790,7 +17805,7 @@
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>371</v>
@@ -17839,7 +17854,7 @@
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>371</v>
@@ -17858,7 +17873,7 @@
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>371</v>
@@ -17877,14 +17892,14 @@
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>371</v>
       </c>
       <c r="G15" s="9"/>
     </row>
-    <row r="16" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A16" s="8" t="s">
         <v>18</v>
       </c>
@@ -17892,12 +17907,16 @@
         <v>19</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>372</v>
+        <v>431</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="10"/>
+      <c r="F16" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>430</v>
+      </c>
     </row>
     <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A17" s="4" t="s">
@@ -17911,7 +17930,7 @@
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>371</v>
@@ -17930,7 +17949,7 @@
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>371</v>
@@ -17949,7 +17968,7 @@
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>371</v>
@@ -17968,7 +17987,7 @@
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>333</v>
@@ -17986,7 +18005,9 @@
         <v>373</v>
       </c>
       <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>424</v>
+      </c>
       <c r="F21" s="4"/>
       <c r="G21" s="9"/>
     </row>
@@ -18002,7 +18023,7 @@
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>371</v>
@@ -18042,7 +18063,7 @@
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>333</v>
@@ -18061,7 +18082,7 @@
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>371</v>
@@ -18080,7 +18101,7 @@
       </c>
       <c r="D26" s="8"/>
       <c r="E26" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>371</v>
@@ -18099,7 +18120,7 @@
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>371</v>
@@ -18139,7 +18160,7 @@
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>333</v>
@@ -18158,7 +18179,7 @@
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>333</v>
@@ -18177,7 +18198,7 @@
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>371</v>
@@ -18196,13 +18217,13 @@
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>371</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -18213,11 +18234,11 @@
         <v>53</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>333</v>
@@ -18232,11 +18253,11 @@
         <v>55</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>333</v>
@@ -18278,7 +18299,7 @@
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F36" s="8" t="s">
         <v>333</v>
@@ -18297,7 +18318,7 @@
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>333</v>
@@ -18316,7 +18337,7 @@
       </c>
       <c r="D38" s="8"/>
       <c r="E38" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F38" s="8" t="s">
         <v>333</v>
@@ -18335,7 +18356,7 @@
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>333</v>
@@ -18367,7 +18388,7 @@
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>333</v>
@@ -18386,7 +18407,7 @@
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F42" s="8" t="s">
         <v>333</v>
@@ -18405,7 +18426,7 @@
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>333</v>
@@ -18424,7 +18445,7 @@
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F44" s="8" t="s">
         <v>371</v>
@@ -18443,7 +18464,7 @@
       </c>
       <c r="D45" s="4"/>
       <c r="E45" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>333</v>
@@ -18481,7 +18502,7 @@
       </c>
       <c r="D47" s="4"/>
       <c r="E47" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>371</v>
@@ -18500,7 +18521,7 @@
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F48" s="8" t="s">
         <v>333</v>
@@ -18519,7 +18540,7 @@
       </c>
       <c r="D49" s="4"/>
       <c r="E49" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>333</v>
@@ -18538,7 +18559,7 @@
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F50" s="8" t="s">
         <v>333</v>
@@ -18574,7 +18595,7 @@
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F52" s="8" t="s">
         <v>333</v>
@@ -18614,13 +18635,13 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F54" s="8" t="s">
         <v>333</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
@@ -18656,13 +18677,13 @@
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F56" s="8" t="s">
         <v>333</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -18677,7 +18698,7 @@
       </c>
       <c r="D57" s="4"/>
       <c r="E57" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F57" s="4" t="s">
         <v>333</v>
@@ -18696,13 +18717,13 @@
       </c>
       <c r="D58" s="8"/>
       <c r="E58" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F58" s="8" t="s">
         <v>333</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -18719,7 +18740,7 @@
         <v>405</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F59" s="4" t="s">
         <v>333</v>
@@ -18738,13 +18759,13 @@
       </c>
       <c r="D60" s="8"/>
       <c r="E60" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F60" s="8" t="s">
         <v>333</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -18755,11 +18776,11 @@
         <v>108</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D61" s="4"/>
       <c r="E61" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>333</v>
@@ -18810,13 +18831,13 @@
       </c>
       <c r="D64" s="8"/>
       <c r="E64" s="8" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="F64" s="8" t="s">
         <v>371</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -18831,7 +18852,7 @@
       </c>
       <c r="D65" s="4"/>
       <c r="E65" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F65" s="4" t="s">
         <v>371</v>
@@ -18859,24 +18880,26 @@
       </c>
       <c r="G66" s="10"/>
     </row>
-    <row r="67" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A67" s="4" t="s">
         <v>119</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C67" s="4" t="s">
-        <v>372</v>
+      <c r="C67" s="16" t="s">
+        <v>431</v>
       </c>
       <c r="D67" s="4"/>
       <c r="E67" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="G67" s="9"/>
+        <v>371</v>
+      </c>
+      <c r="G67" s="10" t="s">
+        <v>430</v>
+      </c>
     </row>
     <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A68" s="8" t="s">
@@ -18890,7 +18913,7 @@
       </c>
       <c r="D68" s="8"/>
       <c r="E68" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F68" s="8" t="s">
         <v>371</v>
@@ -18909,7 +18932,7 @@
       </c>
       <c r="D69" s="4"/>
       <c r="E69" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>371</v>
@@ -18928,7 +18951,7 @@
       </c>
       <c r="D70" s="8"/>
       <c r="E70" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F70" s="8" t="s">
         <v>371</v>
@@ -18947,7 +18970,7 @@
       </c>
       <c r="D71" s="4"/>
       <c r="E71" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>371</v>
@@ -18962,10 +18985,12 @@
         <v>130</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>381</v>
+        <v>432</v>
       </c>
       <c r="D72" s="8"/>
-      <c r="E72" s="8"/>
+      <c r="E72" s="8" t="s">
+        <v>424</v>
+      </c>
       <c r="F72" s="8" t="s">
         <v>333</v>
       </c>
@@ -18983,7 +19008,7 @@
       </c>
       <c r="D73" s="4"/>
       <c r="E73" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F73" s="4" t="s">
         <v>333</v>
@@ -19023,7 +19048,7 @@
       </c>
       <c r="D75" s="4"/>
       <c r="E75" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F75" s="4" t="s">
         <v>333</v>
@@ -19042,7 +19067,7 @@
       </c>
       <c r="D76" s="8"/>
       <c r="E76" s="8" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="F76" s="8" t="s">
         <v>333</v>
@@ -19061,7 +19086,7 @@
       </c>
       <c r="D77" s="4"/>
       <c r="E77" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>333</v>
@@ -19080,7 +19105,7 @@
       </c>
       <c r="D78" s="8"/>
       <c r="E78" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F78" s="8" t="s">
         <v>371</v>
@@ -19118,13 +19143,13 @@
       </c>
       <c r="D80" s="8"/>
       <c r="E80" s="8" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="F80" s="8" t="s">
         <v>371</v>
       </c>
       <c r="G80" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
@@ -19139,7 +19164,7 @@
       </c>
       <c r="D81" s="4"/>
       <c r="E81" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F81" s="4" t="s">
         <v>333</v>
@@ -19154,11 +19179,11 @@
         <v>150</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D82" s="8"/>
       <c r="E82" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F82" s="8"/>
       <c r="G82" s="10"/>
@@ -19175,7 +19200,7 @@
       </c>
       <c r="D83" s="4"/>
       <c r="E83" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F83" s="4"/>
       <c r="G83" s="9"/>
@@ -19188,10 +19213,12 @@
         <v>154</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>381</v>
+        <v>432</v>
       </c>
       <c r="D84" s="8"/>
-      <c r="E84" s="8"/>
+      <c r="E84" s="8" t="s">
+        <v>424</v>
+      </c>
       <c r="F84" s="8" t="s">
         <v>333</v>
       </c>
@@ -19211,7 +19238,7 @@
         <v>391</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F85" s="4" t="s">
         <v>333</v>
@@ -19232,7 +19259,7 @@
         <v>388</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F86" s="8" t="s">
         <v>333</v>
@@ -19253,7 +19280,7 @@
         <v>400</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F87" s="4" t="s">
         <v>333</v>
@@ -19274,7 +19301,7 @@
         <v>407</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F88" s="8" t="s">
         <v>333</v>
@@ -19316,7 +19343,7 @@
         <v>402</v>
       </c>
       <c r="E90" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F90" s="8" t="s">
         <v>333</v>
@@ -19337,7 +19364,7 @@
         <v>394</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F91" s="4" t="s">
         <v>333</v>
@@ -19358,7 +19385,7 @@
         <v>399</v>
       </c>
       <c r="E92" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F92" s="8" t="s">
         <v>333</v>
@@ -19379,7 +19406,7 @@
         <v>393</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F93" s="4" t="s">
         <v>333</v>
@@ -19398,7 +19425,7 @@
       </c>
       <c r="D94" s="8"/>
       <c r="E94" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F94" s="8" t="s">
         <v>333</v>
@@ -19417,13 +19444,13 @@
       </c>
       <c r="D95" s="4"/>
       <c r="E95" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F95" s="4" t="s">
         <v>371</v>
       </c>
       <c r="G95" s="9" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19487,7 +19514,7 @@
       </c>
       <c r="D99" s="4"/>
       <c r="E99" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F99" s="4" t="s">
         <v>333</v>
@@ -19565,7 +19592,7 @@
       </c>
       <c r="D103" s="4"/>
       <c r="E103" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F103" s="4" t="s">
         <v>371</v>
@@ -19599,7 +19626,7 @@
       </c>
       <c r="D105" s="4"/>
       <c r="E105" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F105" s="4" t="s">
         <v>333</v>
@@ -19618,10 +19645,10 @@
       </c>
       <c r="D106" s="8"/>
       <c r="E106" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F106" s="8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="G106" s="10"/>
     </row>
@@ -19656,7 +19683,9 @@
       <c r="C108" s="11" t="s">
         <v>377</v>
       </c>
-      <c r="D108" s="8"/>
+      <c r="D108" s="8" t="s">
+        <v>429</v>
+      </c>
       <c r="E108" s="11" t="s">
         <v>345</v>
       </c>
@@ -19768,7 +19797,7 @@
         <v>406</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F114" s="8" t="s">
         <v>333</v>
@@ -19787,7 +19816,7 @@
       </c>
       <c r="D115" s="4"/>
       <c r="E115" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F115" s="4" t="s">
         <v>333</v>
@@ -19808,7 +19837,7 @@
         <v>397</v>
       </c>
       <c r="E116" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F116" s="8" t="s">
         <v>333</v>
@@ -19829,7 +19858,7 @@
         <v>395</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F117" s="4" t="s">
         <v>333</v>
@@ -19850,7 +19879,7 @@
         <v>404</v>
       </c>
       <c r="E118" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F118" s="8" t="s">
         <v>333</v>
@@ -19871,7 +19900,7 @@
         <v>401</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F119" s="4" t="s">
         <v>333</v>
@@ -19892,13 +19921,13 @@
         <v>396</v>
       </c>
       <c r="E120" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F120" s="8" t="s">
         <v>333</v>
       </c>
       <c r="G120" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
@@ -19915,7 +19944,7 @@
         <v>390</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F121" s="4" t="s">
         <v>333</v>
@@ -19936,7 +19965,7 @@
         <v>389</v>
       </c>
       <c r="E122" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F122" s="8" t="s">
         <v>333</v>
@@ -19957,7 +19986,7 @@
         <v>403</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F123" s="4" t="s">
         <v>333</v>
@@ -19976,7 +20005,7 @@
       </c>
       <c r="D124" s="8"/>
       <c r="E124" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F124" s="8" t="s">
         <v>333</v>
@@ -20012,10 +20041,10 @@
       </c>
       <c r="D126" s="8"/>
       <c r="E126" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F126" s="8" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="G126" s="10"/>
     </row>
@@ -20052,7 +20081,7 @@
       </c>
       <c r="D128" s="8"/>
       <c r="E128" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F128" s="8" t="s">
         <v>371</v>
@@ -20088,7 +20117,7 @@
       </c>
       <c r="D130" s="8"/>
       <c r="E130" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F130" s="8" t="s">
         <v>371</v>
@@ -20107,7 +20136,7 @@
       </c>
       <c r="D131" s="4"/>
       <c r="E131" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F131" s="4" t="s">
         <v>333</v>
@@ -20284,10 +20313,10 @@
       </c>
       <c r="D140" s="8"/>
       <c r="E140" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F140" s="8" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="G140" s="10"/>
     </row>
@@ -20303,7 +20332,7 @@
       </c>
       <c r="D141" s="4"/>
       <c r="E141" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F141" s="4" t="s">
         <v>333</v>
@@ -20322,7 +20351,7 @@
       </c>
       <c r="D142" s="8"/>
       <c r="E142" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F142" s="8" t="s">
         <v>371</v>
@@ -20341,7 +20370,7 @@
       </c>
       <c r="D143" s="4"/>
       <c r="E143" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F143" s="4" t="s">
         <v>333</v>
@@ -20360,7 +20389,7 @@
       </c>
       <c r="D144" s="8"/>
       <c r="E144" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F144" s="8" t="s">
         <v>371</v>
@@ -20379,7 +20408,7 @@
       </c>
       <c r="D145" s="4"/>
       <c r="E145" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F145" s="4" t="s">
         <v>333</v>
@@ -20398,7 +20427,7 @@
       </c>
       <c r="D146" s="8"/>
       <c r="E146" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F146" s="8" t="s">
         <v>333</v>
@@ -20416,7 +20445,7 @@
         <v>373</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F147" s="4" t="s">
         <v>333</v>
@@ -20435,7 +20464,7 @@
       </c>
       <c r="D148" s="8"/>
       <c r="E148" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F148" s="8" t="s">
         <v>333</v>
@@ -20454,7 +20483,7 @@
       </c>
       <c r="D149" s="4"/>
       <c r="E149" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F149" s="4" t="s">
         <v>333</v>
@@ -20473,7 +20502,7 @@
       </c>
       <c r="D150" s="8"/>
       <c r="E150" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F150" s="8" t="s">
         <v>333</v>
@@ -20492,7 +20521,7 @@
       </c>
       <c r="D151" s="4"/>
       <c r="E151" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F151" s="4" t="s">
         <v>333</v>
@@ -20511,7 +20540,7 @@
       </c>
       <c r="D152" s="8"/>
       <c r="E152" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F152" s="8" t="s">
         <v>333</v>
@@ -20530,7 +20559,7 @@
       </c>
       <c r="D153" s="4"/>
       <c r="E153" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F153" s="4" t="s">
         <v>333</v>
@@ -20568,7 +20597,7 @@
       </c>
       <c r="D155" s="4"/>
       <c r="E155" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F155" s="4" t="s">
         <v>333</v>
@@ -20587,7 +20616,7 @@
       </c>
       <c r="D156" s="8"/>
       <c r="E156" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F156" s="8" t="s">
         <v>333</v>
@@ -20606,7 +20635,7 @@
       </c>
       <c r="D157" s="4"/>
       <c r="E157" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F157" s="4" t="s">
         <v>333</v>
@@ -20625,7 +20654,7 @@
       </c>
       <c r="D158" s="8"/>
       <c r="E158" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F158" s="8" t="s">
         <v>333</v>
@@ -20709,7 +20738,7 @@
       </c>
       <c r="D164" s="8"/>
       <c r="E164" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F164" s="8"/>
       <c r="G164" s="10"/>
@@ -20726,7 +20755,7 @@
       </c>
       <c r="D165" s="4"/>
       <c r="E165" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F165" s="4"/>
       <c r="G165" s="9"/>
@@ -20743,7 +20772,7 @@
       </c>
       <c r="D166" s="8"/>
       <c r="E166" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F166" s="8"/>
       <c r="G166" s="10"/>
@@ -20762,7 +20791,7 @@
         <v>358</v>
       </c>
       <c r="E167" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F167" s="4" t="s">
         <v>371</v>
@@ -20781,7 +20810,7 @@
       </c>
       <c r="D168" s="8"/>
       <c r="E168" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F168" s="8" t="s">
         <v>371</v>
@@ -20800,7 +20829,7 @@
       </c>
       <c r="D169" s="4"/>
       <c r="E169" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F169" s="4" t="s">
         <v>371</v>
@@ -20815,11 +20844,11 @@
         <v>326</v>
       </c>
       <c r="C170" s="8" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D170" s="8"/>
       <c r="E170" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F170" s="8"/>
       <c r="G170" s="10"/>

</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA FROTA:CONFERENCIA 23/03 AS 16:15H
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrador\Dropbox\2026\BM COMP 03.26\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CC06A0F-459B-49D2-865D-C95B7C07FB14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{811F2370-AEC9-40B8-99C6-C4DD078C96E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="18" sheetId="6" r:id="rId5"/>
     <sheet name="19" sheetId="7" r:id="rId6"/>
     <sheet name="20" sheetId="8" r:id="rId7"/>
+    <sheet name="23" sheetId="9" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
@@ -29,6 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'18'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'19'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'20'!$A$6:$G$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'23'!$A$6:$G$169</definedName>
   </definedNames>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3883" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4746" uniqueCount="438">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1350,6 +1352,21 @@
   </si>
   <si>
     <t>REGENERAÇÃO</t>
+  </si>
+  <si>
+    <t>22/03/2026 THE X REGENERAÇÃO</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERÊNCIA: 23/03/2026</t>
+  </si>
+  <si>
+    <t>TERESINA / OFICINA</t>
+  </si>
+  <si>
+    <t>VARIOS MUNICIPIOS</t>
+  </si>
+  <si>
+    <t>MUNICIPIOS</t>
   </si>
 </sst>
 </file>
@@ -1945,6 +1962,59 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{020E40E2-BB71-4498-879A-07BDD54A155B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -18070,7 +18140,7 @@
       </c>
       <c r="G24" s="10"/>
     </row>
-    <row r="25" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
       <c r="A25" s="4" t="s">
         <v>36</v>
       </c>
@@ -18078,7 +18148,7 @@
         <v>37</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>373</v>
+        <v>432</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
@@ -18087,7 +18157,9 @@
       <c r="F25" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="G25" s="9"/>
+      <c r="G25" s="9" t="s">
+        <v>433</v>
+      </c>
     </row>
     <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
       <c r="A26" s="8" t="s">
@@ -18887,7 +18959,7 @@
       <c r="B67" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C67" s="16" t="s">
+      <c r="C67" s="4" t="s">
         <v>431</v>
       </c>
       <c r="D67" s="4"/>
@@ -20863,4 +20935,3269 @@
   <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EBD610D-6727-43B3-9A22-6943AE4D8500}">
+  <dimension ref="A1:G169"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
+        <v>434</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D44" s="8"/>
+      <c r="E44" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G54" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G56" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G60" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G67" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F78" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F88" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G95" s="9" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9"/>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E112" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G112" s="9"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C113" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D113" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="10"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G114" s="9"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C115" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D115" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E115" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F115" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G115" s="10"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E116" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G116" s="9"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B117" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C117" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D117" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F117" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G117" s="10"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E118" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G118" s="9"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B119" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C119" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D119" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E119" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F119" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G119" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D120" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E120" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G120" s="9"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D121" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E121" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F121" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G121" s="10"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E122" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G122" s="9"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B123" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C123" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D123" s="8"/>
+      <c r="E123" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F123" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G123" s="10"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
+      <c r="F124" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G124" s="9"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B125" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C125" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D125" s="8"/>
+      <c r="E125" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F125" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="G125" s="10"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E126" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G126" s="9"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C127" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D127" s="8"/>
+      <c r="E127" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F127" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G127" s="10"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+      <c r="F128" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G128" s="9"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="8"/>
+      <c r="E129" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F129" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G129" s="10"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="4"/>
+      <c r="E130" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G130" s="9"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D131" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F131" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G131" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4"/>
+      <c r="F132" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="9"/>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D133" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E133" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F133" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G133" s="10"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D134" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E134" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="9"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C135" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F135" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G135" s="10"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E136" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G136" s="9"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C137" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E137" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="10"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D138" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E138" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="9"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C139" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D139" s="8"/>
+      <c r="E139" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F139" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="G139" s="10"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G140" s="9"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C141" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D141" s="8"/>
+      <c r="E141" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F141" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G141" s="10"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G142" s="9"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B143" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D143" s="8"/>
+      <c r="E143" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F143" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G143" s="10"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G144" s="9"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B145" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C145" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D145" s="8"/>
+      <c r="E145" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F145" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G145" s="10"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C146" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="E146" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G146" s="9"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C147" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F147" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G147" s="10"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D148" s="4"/>
+      <c r="E148" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G148" s="9"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C149" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D149" s="8"/>
+      <c r="E149" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F149" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G149" s="10"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D150" s="4"/>
+      <c r="E150" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G150" s="9"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C151" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D151" s="8"/>
+      <c r="E151" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F151" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G151" s="10"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B152" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C152" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G152" s="9"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C153" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D153" s="8"/>
+      <c r="E153" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F153" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G153" s="10"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C154" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="9"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C155" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D155" s="8"/>
+      <c r="E155" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F155" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G155" s="10"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C156" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G156" s="9"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C157" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F157" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G157" s="10"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D158" s="4"/>
+      <c r="E158" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G158" s="9"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B159" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C159" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D159" s="8"/>
+      <c r="E159" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F159" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G159" s="10"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C160" s="16" t="s">
+        <v>435</v>
+      </c>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F160" s="16" t="s">
+        <v>371</v>
+      </c>
+      <c r="G160" s="9"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B161" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C161" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D161" s="8"/>
+      <c r="E161" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F161" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="G161" s="10"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C162" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D162" s="4"/>
+      <c r="E162" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F162" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="G162" s="9"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B163" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D163" s="8"/>
+      <c r="E163" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G163" s="10"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D164" s="4"/>
+      <c r="E164" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F164" s="16" t="s">
+        <v>372</v>
+      </c>
+      <c r="G164" s="9"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B165" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G165" s="10"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C166" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D166" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E166" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G166" s="9"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B167" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C167" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D167" s="8"/>
+      <c r="E167" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F167" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G167" s="10"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D168" s="4"/>
+      <c r="E168" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G168" s="9"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B169" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="G169" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G169" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ATUALIZAÇÃO PLANILHA FROTA:CONFERENCIA 24/03 AS 10:05H
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrador\Dropbox\2026\BM COMP 03.26\FROTA POTY - CONFERENCIA DIARIA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{811F2370-AEC9-40B8-99C6-C4DD078C96E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE5F775-C96A-4609-8EA4-CFF2794280C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="19" sheetId="7" r:id="rId6"/>
     <sheet name="20" sheetId="8" r:id="rId7"/>
     <sheet name="23" sheetId="9" r:id="rId8"/>
+    <sheet name="24" sheetId="10" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
@@ -31,6 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'19'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'20'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'23'!$A$6:$G$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'24'!$A$6:$G$169</definedName>
   </definedNames>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -50,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4746" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5608" uniqueCount="439">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1367,6 +1369,9 @@
   </si>
   <si>
     <t>MUNICIPIOS</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERÊNCIA: 24/03/2026</t>
   </si>
 </sst>
 </file>
@@ -1520,7 +1525,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1560,9 +1565,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2015,6 +2017,59 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DCD33EF-1BA6-4735-8211-33C84B58AD08}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -24005,14 +24060,14 @@
       <c r="B160" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="C160" s="16" t="s">
+      <c r="C160" s="4" t="s">
         <v>435</v>
       </c>
       <c r="D160" s="4"/>
       <c r="E160" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="F160" s="16" t="s">
+      <c r="F160" s="4" t="s">
         <v>371</v>
       </c>
       <c r="G160" s="9"/>
@@ -24050,7 +24105,7 @@
       <c r="E162" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="F162" s="16" t="s">
+      <c r="F162" s="4" t="s">
         <v>437</v>
       </c>
       <c r="G162" s="9"/>
@@ -24088,7 +24143,3272 @@
       <c r="E164" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="F164" s="16" t="s">
+      <c r="F164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G164" s="9"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B165" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G165" s="10"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C166" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D166" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E166" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G166" s="9"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B167" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C167" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D167" s="8"/>
+      <c r="E167" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F167" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G167" s="10"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D168" s="4"/>
+      <c r="E168" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G168" s="9"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B169" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="G169" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G169" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B29DB5-D8F8-4052-92CC-E31F91B45F6C}">
+  <dimension ref="A1:G169"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
+        <v>438</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D44" s="8"/>
+      <c r="E44" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G54" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G56" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G60" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G67" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F78" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F88" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G95" s="9" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9"/>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E112" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G112" s="9"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C113" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D113" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="10"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G114" s="9"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C115" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D115" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E115" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F115" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G115" s="10"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E116" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G116" s="9"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B117" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C117" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D117" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F117" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G117" s="10"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E118" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G118" s="9"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B119" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C119" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D119" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E119" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F119" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G119" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D120" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E120" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G120" s="9"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D121" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E121" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F121" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G121" s="10"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E122" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G122" s="9"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B123" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C123" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D123" s="8"/>
+      <c r="E123" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F123" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G123" s="10"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
+      <c r="F124" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G124" s="9"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B125" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C125" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D125" s="8"/>
+      <c r="E125" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F125" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="G125" s="10"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E126" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G126" s="9"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C127" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D127" s="8"/>
+      <c r="E127" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F127" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G127" s="10"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+      <c r="F128" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G128" s="9"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="8"/>
+      <c r="E129" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F129" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G129" s="10"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="4"/>
+      <c r="E130" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G130" s="9"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D131" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F131" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G131" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4"/>
+      <c r="F132" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="9"/>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D133" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E133" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F133" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G133" s="10"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D134" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E134" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="9"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C135" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F135" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G135" s="10"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E136" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G136" s="9"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C137" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E137" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="10"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D138" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E138" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="9"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C139" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D139" s="8"/>
+      <c r="E139" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F139" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="G139" s="10"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G140" s="9"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C141" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D141" s="8"/>
+      <c r="E141" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F141" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G141" s="10"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G142" s="9"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B143" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D143" s="8"/>
+      <c r="E143" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F143" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G143" s="10"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G144" s="9"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B145" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C145" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D145" s="8"/>
+      <c r="E145" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F145" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G145" s="10"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C146" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="E146" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G146" s="9"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C147" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F147" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G147" s="10"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D148" s="4"/>
+      <c r="E148" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G148" s="9"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C149" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D149" s="8"/>
+      <c r="E149" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F149" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G149" s="10"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D150" s="4"/>
+      <c r="E150" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G150" s="9"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C151" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D151" s="8"/>
+      <c r="E151" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F151" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G151" s="10"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B152" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C152" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G152" s="9"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C153" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D153" s="8"/>
+      <c r="E153" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F153" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G153" s="10"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C154" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="9"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C155" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D155" s="8"/>
+      <c r="E155" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F155" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G155" s="10"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C156" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G156" s="9"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C157" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F157" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G157" s="10"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D158" s="4"/>
+      <c r="E158" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G158" s="9"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B159" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C159" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D159" s="8"/>
+      <c r="E159" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F159" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G159" s="10"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C160" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F160" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G160" s="9"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B161" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C161" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D161" s="8"/>
+      <c r="E161" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F161" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="G161" s="10"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C162" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D162" s="4"/>
+      <c r="E162" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F162" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="G162" s="9"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B163" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D163" s="8"/>
+      <c r="E163" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G163" s="10"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D164" s="4"/>
+      <c r="E164" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F164" s="4" t="s">
         <v>372</v>
       </c>
       <c r="G164" s="9"/>

</xml_diff>

<commit_message>
ATUALIZAÇÃO FROTA: 25/03 AS 11:30
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE5F775-C96A-4609-8EA4-CFF2794280C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E423B82-CBC6-4AAC-8785-A5214129C66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,7 @@
     <sheet name="20" sheetId="8" r:id="rId7"/>
     <sheet name="23" sheetId="9" r:id="rId8"/>
     <sheet name="24" sheetId="10" r:id="rId9"/>
+    <sheet name="25" sheetId="11" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
@@ -33,6 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'20'!$A$6:$G$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'23'!$A$6:$G$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'24'!$A$6:$G$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'25'!$A$6:$G$169</definedName>
   </definedNames>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -52,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5608" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6470" uniqueCount="441">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1372,6 +1374,12 @@
   </si>
   <si>
     <t>DATA DA CONFERÊNCIA: 24/03/2026</t>
+  </si>
+  <si>
+    <t>MADEIRO</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERÊNCIA: 25/03/2026</t>
   </si>
 </sst>
 </file>
@@ -1614,6 +1622,59 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB79E929-BC57-4760-ACC1-316EEF0866B7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12FF9EE0-3477-45CD-BCDC-9275A9B48C56}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4774,6 +4835,3271 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{978016E3-D942-4881-BB1F-C8ACBDC3D27C}">
+  <dimension ref="A1:G169"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
+        <v>438</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D44" s="8"/>
+      <c r="E44" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G54" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G56" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G60" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G67" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F78" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F88" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G95" s="9" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9"/>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E112" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G112" s="9"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C113" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D113" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="10"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G114" s="9"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C115" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D115" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E115" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F115" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G115" s="10"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E116" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G116" s="9"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B117" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C117" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D117" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F117" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G117" s="10"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E118" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G118" s="9"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B119" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C119" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D119" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E119" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F119" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G119" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D120" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E120" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G120" s="9"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D121" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E121" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F121" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G121" s="10"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E122" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G122" s="9"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B123" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C123" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D123" s="8"/>
+      <c r="E123" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F123" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G123" s="10"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
+      <c r="F124" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G124" s="9"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B125" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C125" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D125" s="8"/>
+      <c r="E125" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F125" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="G125" s="10"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E126" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G126" s="9"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C127" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D127" s="8"/>
+      <c r="E127" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F127" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G127" s="10"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+      <c r="F128" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G128" s="9"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="8"/>
+      <c r="E129" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F129" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G129" s="10"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="4"/>
+      <c r="E130" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G130" s="9"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D131" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F131" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G131" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4"/>
+      <c r="F132" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="9"/>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D133" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E133" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F133" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G133" s="10"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D134" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E134" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="9"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C135" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F135" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G135" s="10"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E136" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G136" s="9"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C137" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E137" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="10"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D138" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E138" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="9"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C139" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D139" s="8"/>
+      <c r="E139" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F139" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="G139" s="10"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G140" s="9"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C141" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D141" s="8"/>
+      <c r="E141" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F141" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G141" s="10"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G142" s="9"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B143" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D143" s="8"/>
+      <c r="E143" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F143" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G143" s="10"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G144" s="9"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B145" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C145" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D145" s="8"/>
+      <c r="E145" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F145" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G145" s="10"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C146" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="E146" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G146" s="9"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C147" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F147" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G147" s="10"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D148" s="4"/>
+      <c r="E148" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G148" s="9"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C149" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D149" s="8"/>
+      <c r="E149" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F149" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G149" s="10"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D150" s="4"/>
+      <c r="E150" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G150" s="9"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C151" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D151" s="8"/>
+      <c r="E151" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F151" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G151" s="10"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B152" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C152" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G152" s="9"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C153" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D153" s="8"/>
+      <c r="E153" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F153" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G153" s="10"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C154" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="9"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C155" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D155" s="8"/>
+      <c r="E155" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F155" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G155" s="10"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C156" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G156" s="9"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C157" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F157" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G157" s="10"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D158" s="4"/>
+      <c r="E158" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G158" s="9"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B159" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C159" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D159" s="8"/>
+      <c r="E159" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F159" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G159" s="10"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C160" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F160" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G160" s="9"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B161" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C161" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D161" s="8"/>
+      <c r="E161" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F161" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="G161" s="10"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C162" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D162" s="4"/>
+      <c r="E162" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F162" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="G162" s="9"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B163" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D163" s="8"/>
+      <c r="E163" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G163" s="10"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D164" s="4"/>
+      <c r="E164" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G164" s="9"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B165" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G165" s="10"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C166" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D166" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E166" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G166" s="9"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B167" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C167" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D167" s="8"/>
+      <c r="E167" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F167" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G167" s="10"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D168" s="4"/>
+      <c r="E168" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G168" s="9"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B169" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="G169" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G169" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CD45BB0-E105-48DD-9525-BAF52D0E0BB5}">
   <dimension ref="A1:G170"/>
@@ -24304,7 +27630,7 @@
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
@@ -25732,7 +29058,7 @@
         <v>144</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>376</v>
+        <v>439</v>
       </c>
       <c r="D79" s="4"/>
       <c r="E79" s="4" t="s">

</xml_diff>

<commit_message>
ATUALIZAÇÃO FROTA: 26/03 AS 09h
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E423B82-CBC6-4AAC-8785-A5214129C66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F377C62B-8C09-4C22-9D6D-A8D537D16D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="23" sheetId="9" r:id="rId8"/>
     <sheet name="24" sheetId="10" r:id="rId9"/>
     <sheet name="25" sheetId="11" r:id="rId10"/>
+    <sheet name="26" sheetId="12" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
@@ -35,6 +36,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'23'!$A$6:$G$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'24'!$A$6:$G$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'25'!$A$6:$G$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'26'!$A$6:$G$169</definedName>
   </definedNames>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -54,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6470" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7335" uniqueCount="443">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1380,6 +1382,12 @@
   </si>
   <si>
     <t>DATA DA CONFERÊNCIA: 25/03/2026</t>
+  </si>
+  <si>
+    <t>PI 240 / ANTÔNIO ALMEIDA X CADOZ 25/03</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERÊNCIA: 26/03/2026</t>
   </si>
 </sst>
 </file>
@@ -1675,6 +1683,59 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12FF9EE0-3477-45CD-BCDC-9275A9B48C56}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8EC091AC-9FCB-421B-AAB9-98E93465B2A9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4882,7 +4943,7 @@
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
@@ -6862,7 +6923,7 @@
         <v>200</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>340</v>
@@ -6873,7 +6934,3276 @@
       <c r="F107" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="G107" s="9"/>
+      <c r="G107" s="4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9"/>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E112" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G112" s="9"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C113" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D113" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="10"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G114" s="9"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C115" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D115" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E115" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F115" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G115" s="10"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E116" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G116" s="9"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B117" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C117" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D117" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F117" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G117" s="10"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E118" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G118" s="9"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B119" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C119" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D119" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E119" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F119" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G119" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D120" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E120" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G120" s="9"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D121" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E121" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F121" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G121" s="10"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E122" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G122" s="9"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B123" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C123" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D123" s="8"/>
+      <c r="E123" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F123" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G123" s="10"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
+      <c r="F124" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G124" s="9"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B125" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C125" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D125" s="8"/>
+      <c r="E125" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F125" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="G125" s="10"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E126" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G126" s="9"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C127" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D127" s="8"/>
+      <c r="E127" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F127" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G127" s="10"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+      <c r="F128" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G128" s="9"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="8"/>
+      <c r="E129" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F129" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G129" s="10"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="4"/>
+      <c r="E130" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G130" s="9"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D131" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F131" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G131" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4"/>
+      <c r="F132" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="9"/>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D133" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E133" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F133" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G133" s="10"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D134" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E134" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="9"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C135" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F135" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G135" s="10"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E136" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G136" s="9"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C137" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E137" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="10"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D138" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E138" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="9"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C139" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D139" s="8"/>
+      <c r="E139" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F139" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="G139" s="10"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G140" s="9"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C141" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D141" s="8"/>
+      <c r="E141" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F141" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G141" s="10"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G142" s="9"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B143" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D143" s="8"/>
+      <c r="E143" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F143" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G143" s="10"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G144" s="9"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B145" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C145" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D145" s="8"/>
+      <c r="E145" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F145" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G145" s="10"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C146" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="E146" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G146" s="9"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C147" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F147" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G147" s="10"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D148" s="4"/>
+      <c r="E148" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G148" s="9"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C149" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D149" s="8"/>
+      <c r="E149" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F149" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G149" s="10"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D150" s="4"/>
+      <c r="E150" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G150" s="9"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C151" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D151" s="8"/>
+      <c r="E151" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F151" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G151" s="10"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B152" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C152" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G152" s="9"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C153" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D153" s="8"/>
+      <c r="E153" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F153" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G153" s="10"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C154" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="9"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C155" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D155" s="8"/>
+      <c r="E155" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F155" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G155" s="10"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C156" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G156" s="9"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C157" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F157" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G157" s="10"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D158" s="4"/>
+      <c r="E158" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G158" s="9"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B159" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C159" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D159" s="8"/>
+      <c r="E159" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F159" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G159" s="10"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C160" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F160" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G160" s="9"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B161" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C161" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D161" s="8"/>
+      <c r="E161" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F161" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="G161" s="10"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C162" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D162" s="4"/>
+      <c r="E162" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F162" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="G162" s="9"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B163" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D163" s="8"/>
+      <c r="E163" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G163" s="10"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D164" s="4"/>
+      <c r="E164" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G164" s="9"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B165" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G165" s="10"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C166" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D166" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E166" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G166" s="9"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B167" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C167" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D167" s="8"/>
+      <c r="E167" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F167" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G167" s="10"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D168" s="4"/>
+      <c r="E168" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G168" s="9"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B169" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="G169" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G169" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A773D76B-9A57-4A17-B38B-FC3618FF50B6}">
+  <dimension ref="A1:G169"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
+        <v>442</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D44" s="8"/>
+      <c r="E44" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G54" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G56" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G60" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G67" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F78" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F88" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G95" s="9" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="4" t="s">
+        <v>441</v>
+      </c>
     </row>
     <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="8" t="s">
@@ -27630,7 +30960,7 @@
     <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
@@ -29610,7 +32940,7 @@
         <v>200</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>340</v>
@@ -29621,7 +32951,9 @@
       <c r="F107" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="G107" s="9"/>
+      <c r="G107" s="4" t="s">
+        <v>441</v>
+      </c>
     </row>
     <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="8" t="s">

</xml_diff>

<commit_message>
ATUALIZAÇÃO FROTA: 27/03 10:30
</commit_message>
<xml_diff>
--- a/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
+++ b/FROTA POTY - CONFERENCIA DIARIA/CONFERENCIA_FROTA_MARÇO.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\FROTA POTY - CONFERENCIA DIARIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F377C62B-8C09-4C22-9D6D-A8D537D16D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D692D363-3218-4B06-925E-53090A663486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="2" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="24" sheetId="10" r:id="rId9"/>
     <sheet name="25" sheetId="11" r:id="rId10"/>
     <sheet name="26" sheetId="12" r:id="rId11"/>
+    <sheet name="27" sheetId="13" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'12'!$A$6:$G$170</definedName>
@@ -37,6 +38,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'24'!$A$6:$G$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'25'!$A$6:$G$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'26'!$A$6:$G$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'27'!$A$6:$G$169</definedName>
   </definedNames>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -56,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7335" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8198" uniqueCount="444">
   <si>
     <t xml:space="preserve">01.001 </t>
   </si>
@@ -1388,6 +1390,9 @@
   </si>
   <si>
     <t>DATA DA CONFERÊNCIA: 26/03/2026</t>
+  </si>
+  <si>
+    <t>DATA DA CONFERÊNCIA: 27/03/2026</t>
   </si>
 </sst>
 </file>
@@ -1736,6 +1741,59 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8EC091AC-9FCB-421B-AAB9-98E93465B2A9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="0"/>
+          <a:ext cx="1200150" cy="369277"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>666751</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{019E2775-48A9-48E3-9E56-E54F352D4931}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -11430,6 +11488,3273 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C69EBBB-CB8A-425F-A9C4-4DCA615A93A4}">
+  <dimension ref="A1:G169"/>
+  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="5"/>
+    <col min="2" max="2" width="49.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
+        <v>443</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F21" s="4"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="7" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A39" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A42" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A43" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A44" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D44" s="8"/>
+      <c r="E44" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A45" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G46" s="10">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A48" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A49" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A50" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A52" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A54" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G54" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G56" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A58" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A60" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G60" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A61" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A62" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G62" s="10"/>
+    </row>
+    <row r="63" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A63" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A64" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F64" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G64" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A66" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G66" s="10"/>
+    </row>
+    <row r="67" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A67" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G67" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A68" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G68" s="10"/>
+    </row>
+    <row r="69" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A70" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="10"/>
+    </row>
+    <row r="71" spans="1:7" s="7" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A72" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A73" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A74" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G74" s="10"/>
+    </row>
+    <row r="75" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G76" s="10"/>
+    </row>
+    <row r="77" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A77" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A78" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F78" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A80" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F80" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G80" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A81" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A82" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F82" s="8"/>
+      <c r="G82" s="10"/>
+    </row>
+    <row r="83" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A83" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F83" s="4"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" ht="9" x14ac:dyDescent="0.15">
+      <c r="A84" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F84" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.15">
+      <c r="A85" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F88" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G92" s="10"/>
+    </row>
+    <row r="93" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G95" s="9" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G96" s="10"/>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G98" s="10"/>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G107" s="4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D108" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="E108" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G109" s="9"/>
+    </row>
+    <row r="110" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G110" s="10"/>
+    </row>
+    <row r="111" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E112" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G112" s="9"/>
+    </row>
+    <row r="113" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C113" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D113" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G113" s="10"/>
+    </row>
+    <row r="114" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G114" s="9"/>
+    </row>
+    <row r="115" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C115" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D115" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E115" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F115" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G115" s="10"/>
+    </row>
+    <row r="116" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="E116" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G116" s="9"/>
+    </row>
+    <row r="117" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B117" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C117" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D117" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F117" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G117" s="10"/>
+    </row>
+    <row r="118" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E118" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G118" s="9"/>
+    </row>
+    <row r="119" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B119" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C119" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D119" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E119" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F119" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G119" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D120" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E120" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G120" s="9"/>
+    </row>
+    <row r="121" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D121" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E121" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="F121" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G121" s="10"/>
+    </row>
+    <row r="122" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D122" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="E122" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G122" s="9"/>
+    </row>
+    <row r="123" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B123" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C123" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D123" s="8"/>
+      <c r="E123" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F123" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G123" s="10"/>
+    </row>
+    <row r="124" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
+      <c r="F124" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G124" s="9"/>
+    </row>
+    <row r="125" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B125" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C125" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D125" s="8"/>
+      <c r="E125" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F125" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="G125" s="10"/>
+    </row>
+    <row r="126" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A126" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E126" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G126" s="9"/>
+    </row>
+    <row r="127" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A127" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C127" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D127" s="8"/>
+      <c r="E127" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F127" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G127" s="10"/>
+    </row>
+    <row r="128" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A128" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+      <c r="F128" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G128" s="9"/>
+    </row>
+    <row r="129" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A129" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D129" s="8"/>
+      <c r="E129" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F129" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G129" s="10"/>
+    </row>
+    <row r="130" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D130" s="4"/>
+      <c r="E130" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G130" s="9"/>
+    </row>
+    <row r="131" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A131" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="D131" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F131" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G131" s="10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A132" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4"/>
+      <c r="F132" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G132" s="9"/>
+    </row>
+    <row r="133" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A133" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D133" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E133" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="F133" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G133" s="10"/>
+    </row>
+    <row r="134" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A134" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D134" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E134" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G134" s="9"/>
+    </row>
+    <row r="135" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C135" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F135" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G135" s="10"/>
+    </row>
+    <row r="136" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E136" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G136" s="9"/>
+    </row>
+    <row r="137" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A137" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C137" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D137" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="E137" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="F137" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G137" s="10"/>
+    </row>
+    <row r="138" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A138" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D138" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E138" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G138" s="9"/>
+    </row>
+    <row r="139" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A139" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C139" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D139" s="8"/>
+      <c r="E139" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F139" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="G139" s="10"/>
+    </row>
+    <row r="140" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A140" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G140" s="9"/>
+    </row>
+    <row r="141" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A141" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C141" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D141" s="8"/>
+      <c r="E141" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F141" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G141" s="10"/>
+    </row>
+    <row r="142" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G142" s="9"/>
+    </row>
+    <row r="143" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A143" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B143" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D143" s="8"/>
+      <c r="E143" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F143" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G143" s="10"/>
+    </row>
+    <row r="144" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G144" s="9"/>
+    </row>
+    <row r="145" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B145" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C145" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D145" s="8"/>
+      <c r="E145" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F145" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G145" s="10"/>
+    </row>
+    <row r="146" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A146" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C146" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="E146" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G146" s="9"/>
+    </row>
+    <row r="147" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A147" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C147" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F147" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G147" s="10"/>
+    </row>
+    <row r="148" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A148" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D148" s="4"/>
+      <c r="E148" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G148" s="9"/>
+    </row>
+    <row r="149" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A149" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="C149" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D149" s="8"/>
+      <c r="E149" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F149" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G149" s="10"/>
+    </row>
+    <row r="150" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A150" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D150" s="4"/>
+      <c r="E150" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G150" s="9"/>
+    </row>
+    <row r="151" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A151" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C151" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D151" s="8"/>
+      <c r="E151" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F151" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G151" s="10"/>
+    </row>
+    <row r="152" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A152" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B152" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C152" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G152" s="9"/>
+    </row>
+    <row r="153" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A153" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="C153" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="D153" s="8"/>
+      <c r="E153" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F153" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G153" s="10"/>
+    </row>
+    <row r="154" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A154" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C154" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G154" s="9"/>
+    </row>
+    <row r="155" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C155" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D155" s="8"/>
+      <c r="E155" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F155" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G155" s="10"/>
+    </row>
+    <row r="156" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A156" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C156" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G156" s="9"/>
+    </row>
+    <row r="157" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A157" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C157" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F157" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="G157" s="10"/>
+    </row>
+    <row r="158" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A158" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D158" s="4"/>
+      <c r="E158" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G158" s="9"/>
+    </row>
+    <row r="159" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A159" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B159" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C159" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="D159" s="8"/>
+      <c r="E159" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F159" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G159" s="10"/>
+    </row>
+    <row r="160" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A160" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C160" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F160" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G160" s="9"/>
+    </row>
+    <row r="161" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A161" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B161" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C161" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D161" s="8"/>
+      <c r="E161" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F161" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="G161" s="10"/>
+    </row>
+    <row r="162" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A162" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C162" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D162" s="4"/>
+      <c r="E162" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F162" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="G162" s="9"/>
+    </row>
+    <row r="163" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A163" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="B163" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D163" s="8"/>
+      <c r="E163" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F163" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G163" s="10"/>
+    </row>
+    <row r="164" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A164" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D164" s="4"/>
+      <c r="E164" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F164" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G164" s="9"/>
+    </row>
+    <row r="165" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A165" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B165" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F165" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="G165" s="10"/>
+    </row>
+    <row r="166" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A166" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C166" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D166" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E166" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G166" s="9"/>
+    </row>
+    <row r="167" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A167" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B167" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C167" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="D167" s="8"/>
+      <c r="E167" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F167" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="G167" s="10"/>
+    </row>
+    <row r="168" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A168" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D168" s="4"/>
+      <c r="E168" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G168" s="9"/>
+    </row>
+    <row r="169" spans="1:7" s="7" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A169" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B169" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F169" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="G169" s="10"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G169" xr:uid="{E0D125D0-C45E-4DC2-832B-9FB94130ECD7}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" scale="80" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CD45BB0-E105-48DD-9525-BAF52D0E0BB5}">
   <dimension ref="A1:G170"/>

</xml_diff>